<commit_message>
fix:hci template date size
</commit_message>
<xml_diff>
--- a/SupervisorMobility.API/DataAccess/Templates/HCI Template.xlsx
+++ b/SupervisorMobility.API/DataAccess/Templates/HCI Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\job\Supervisor app\Server\SupervisorMobility.API\DataAccess\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FD4DFAB-3802-427A-9E37-0B2803011137}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C8C37F8-521F-4A35-A1C9-FC777A35B168}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31695" yWindow="3210" windowWidth="21840" windowHeight="15285" xr2:uid="{04842937-1B74-41D6-BD72-7F55AB7A96D5}"/>
+    <workbookView xWindow="38775" yWindow="3420" windowWidth="24360" windowHeight="15840" xr2:uid="{04842937-1B74-41D6-BD72-7F55AB7A96D5}"/>
   </bookViews>
   <sheets>
     <sheet name="HCI" sheetId="1" r:id="rId1"/>
@@ -910,7 +910,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -975,7 +975,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -986,7 +985,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1017,6 +1015,141 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1071,140 +1204,14 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1766,105 +1773,105 @@
         <v>0</v>
       </c>
       <c r="B3" s="3"/>
-      <c r="C3" s="46" t="s">
+      <c r="C3" s="89" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="47"/>
-      <c r="E3" s="48"/>
-      <c r="F3" s="49"/>
-      <c r="G3" s="50" t="s">
+      <c r="D3" s="90"/>
+      <c r="E3" s="91"/>
+      <c r="F3" s="92"/>
+      <c r="G3" s="93" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="51"/>
-      <c r="I3" s="51"/>
-      <c r="J3" s="52"/>
-      <c r="K3" s="52"/>
-      <c r="L3" s="53"/>
-      <c r="M3" s="54" t="s">
+      <c r="H3" s="94"/>
+      <c r="I3" s="94"/>
+      <c r="J3" s="95"/>
+      <c r="K3" s="95"/>
+      <c r="L3" s="96"/>
+      <c r="M3" s="97" t="s">
         <v>3</v>
       </c>
-      <c r="N3" s="55"/>
-      <c r="O3" s="55"/>
-      <c r="P3" s="55"/>
-      <c r="Q3" s="55"/>
-      <c r="R3" s="56"/>
+      <c r="N3" s="98"/>
+      <c r="O3" s="98"/>
+      <c r="P3" s="98"/>
+      <c r="Q3" s="98"/>
+      <c r="R3" s="99"/>
     </row>
     <row r="4" spans="1:18" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="44"/>
+      <c r="B4" s="42"/>
       <c r="C4" s="5" t="s">
         <v>5</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="7"/>
-      <c r="F4" s="45"/>
-      <c r="G4" s="59" t="s">
+      <c r="F4" s="43"/>
+      <c r="G4" s="102" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="60"/>
-      <c r="I4" s="60"/>
-      <c r="J4" s="61"/>
-      <c r="K4" s="61"/>
-      <c r="L4" s="62"/>
-      <c r="M4" s="63"/>
-      <c r="N4" s="63"/>
-      <c r="O4" s="63"/>
-      <c r="P4" s="63"/>
-      <c r="Q4" s="63"/>
-      <c r="R4" s="57"/>
+      <c r="H4" s="103"/>
+      <c r="I4" s="103"/>
+      <c r="J4" s="104"/>
+      <c r="K4" s="104"/>
+      <c r="L4" s="105"/>
+      <c r="M4" s="106"/>
+      <c r="N4" s="106"/>
+      <c r="O4" s="106"/>
+      <c r="P4" s="106"/>
+      <c r="Q4" s="106"/>
+      <c r="R4" s="100"/>
     </row>
     <row r="5" spans="1:18" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="77" t="s">
+      <c r="A5" s="81" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="77"/>
-      <c r="C5" s="77" t="s">
+      <c r="B5" s="81"/>
+      <c r="C5" s="81" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="77"/>
-      <c r="E5" s="77"/>
-      <c r="F5" s="77"/>
-      <c r="G5" s="77"/>
-      <c r="H5" s="77"/>
-      <c r="I5" s="77"/>
-      <c r="J5" s="77"/>
-      <c r="K5" s="77"/>
-      <c r="L5" s="77"/>
-      <c r="R5" s="57"/>
+      <c r="D5" s="81"/>
+      <c r="E5" s="81"/>
+      <c r="F5" s="81"/>
+      <c r="G5" s="81"/>
+      <c r="H5" s="81"/>
+      <c r="I5" s="81"/>
+      <c r="J5" s="81"/>
+      <c r="K5" s="81"/>
+      <c r="L5" s="81"/>
+      <c r="R5" s="100"/>
     </row>
     <row r="6" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="78" t="s">
+      <c r="A6" s="82" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="79"/>
-      <c r="D6" s="78" t="s">
+      <c r="B6" s="83"/>
+      <c r="D6" s="82" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="82"/>
-      <c r="F6" s="82"/>
-      <c r="G6" s="82"/>
-      <c r="H6" s="82"/>
-      <c r="I6" s="82"/>
-      <c r="J6" s="82"/>
-      <c r="K6" s="82"/>
-      <c r="L6" s="79"/>
-      <c r="R6" s="57"/>
+      <c r="E6" s="86"/>
+      <c r="F6" s="86"/>
+      <c r="G6" s="86"/>
+      <c r="H6" s="86"/>
+      <c r="I6" s="86"/>
+      <c r="J6" s="86"/>
+      <c r="K6" s="86"/>
+      <c r="L6" s="83"/>
+      <c r="R6" s="100"/>
     </row>
     <row r="7" spans="1:18" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="80"/>
-      <c r="B7" s="81"/>
-      <c r="D7" s="80"/>
-      <c r="E7" s="83"/>
-      <c r="F7" s="83"/>
-      <c r="G7" s="83"/>
-      <c r="H7" s="83"/>
-      <c r="I7" s="83"/>
-      <c r="J7" s="83"/>
-      <c r="K7" s="83"/>
-      <c r="L7" s="81"/>
-      <c r="R7" s="58"/>
+      <c r="A7" s="84"/>
+      <c r="B7" s="85"/>
+      <c r="D7" s="84"/>
+      <c r="E7" s="87"/>
+      <c r="F7" s="87"/>
+      <c r="G7" s="87"/>
+      <c r="H7" s="87"/>
+      <c r="I7" s="87"/>
+      <c r="J7" s="87"/>
+      <c r="K7" s="87"/>
+      <c r="L7" s="85"/>
+      <c r="R7" s="101"/>
     </row>
     <row r="8" spans="1:18" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="8" t="s">
@@ -1882,33 +1889,33 @@
       <c r="F8" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="G8" s="84" t="s">
+      <c r="G8" s="69" t="s">
         <v>16</v>
       </c>
-      <c r="H8" s="85"/>
-      <c r="I8" s="86"/>
-      <c r="J8" s="84" t="s">
+      <c r="H8" s="70"/>
+      <c r="I8" s="68"/>
+      <c r="J8" s="69" t="s">
         <v>17</v>
       </c>
-      <c r="K8" s="85"/>
-      <c r="L8" s="87"/>
+      <c r="K8" s="70"/>
+      <c r="L8" s="88"/>
     </row>
     <row r="9" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="24"/>
-      <c r="B9" s="25"/>
-      <c r="D9" s="33"/>
-      <c r="E9" s="34"/>
-      <c r="F9" s="34"/>
-      <c r="G9" s="64"/>
-      <c r="H9" s="65"/>
-      <c r="I9" s="76"/>
-      <c r="J9" s="64"/>
-      <c r="K9" s="65"/>
-      <c r="L9" s="66"/>
-      <c r="N9" s="67" t="s">
+      <c r="A9" s="109"/>
+      <c r="B9" s="24"/>
+      <c r="D9" s="31"/>
+      <c r="E9" s="32"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="78"/>
+      <c r="H9" s="71"/>
+      <c r="I9" s="59"/>
+      <c r="J9" s="78"/>
+      <c r="K9" s="71"/>
+      <c r="L9" s="72"/>
+      <c r="N9" s="79" t="s">
         <v>18</v>
       </c>
-      <c r="O9" s="68"/>
+      <c r="O9" s="80"/>
       <c r="P9" s="13" t="s">
         <v>19</v>
       </c>
@@ -1916,215 +1923,215 @@
       <c r="R9" s="15"/>
     </row>
     <row r="10" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="26"/>
-      <c r="B10" s="27"/>
+      <c r="A10" s="25"/>
+      <c r="B10" s="26"/>
       <c r="C10" s="16"/>
-      <c r="D10" s="35"/>
-      <c r="E10" s="36"/>
-      <c r="F10" s="37"/>
-      <c r="G10" s="69"/>
-      <c r="H10" s="70"/>
-      <c r="I10" s="71"/>
-      <c r="J10" s="72"/>
-      <c r="K10" s="73"/>
-      <c r="L10" s="74"/>
+      <c r="D10" s="33"/>
+      <c r="E10" s="34"/>
+      <c r="F10" s="35"/>
+      <c r="G10" s="73"/>
+      <c r="H10" s="74"/>
+      <c r="I10" s="75"/>
+      <c r="J10" s="76"/>
+      <c r="K10" s="48"/>
+      <c r="L10" s="49"/>
       <c r="M10" s="17"/>
-      <c r="N10" s="75"/>
-      <c r="O10" s="76"/>
-      <c r="P10" s="64"/>
-      <c r="Q10" s="65"/>
-      <c r="R10" s="66"/>
+      <c r="N10" s="58"/>
+      <c r="O10" s="59"/>
+      <c r="P10" s="78"/>
+      <c r="Q10" s="71"/>
+      <c r="R10" s="72"/>
     </row>
     <row r="11" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="26"/>
-      <c r="B11" s="27"/>
+      <c r="A11" s="25"/>
+      <c r="B11" s="26"/>
       <c r="C11" s="16"/>
-      <c r="D11" s="35"/>
-      <c r="E11" s="36"/>
-      <c r="F11" s="38"/>
-      <c r="G11" s="69"/>
-      <c r="H11" s="70"/>
-      <c r="I11" s="71"/>
-      <c r="J11" s="72"/>
-      <c r="K11" s="73"/>
-      <c r="L11" s="74"/>
+      <c r="D11" s="33"/>
+      <c r="E11" s="34"/>
+      <c r="F11" s="36"/>
+      <c r="G11" s="73"/>
+      <c r="H11" s="74"/>
+      <c r="I11" s="75"/>
+      <c r="J11" s="76"/>
+      <c r="K11" s="48"/>
+      <c r="L11" s="49"/>
       <c r="M11" s="18"/>
-      <c r="N11" s="88"/>
-      <c r="O11" s="89"/>
-      <c r="P11" s="72" t="s">
+      <c r="N11" s="44"/>
+      <c r="O11" s="45"/>
+      <c r="P11" s="76" t="s">
         <v>20</v>
       </c>
-      <c r="Q11" s="73"/>
-      <c r="R11" s="74"/>
+      <c r="Q11" s="48"/>
+      <c r="R11" s="49"/>
     </row>
     <row r="12" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="28" t="s">
+      <c r="A12" s="107" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="29"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="39"/>
-      <c r="F12" s="39"/>
-      <c r="G12" s="69"/>
-      <c r="H12" s="70"/>
-      <c r="I12" s="71"/>
-      <c r="J12" s="72"/>
-      <c r="K12" s="73"/>
-      <c r="L12" s="74"/>
-      <c r="N12" s="88"/>
-      <c r="O12" s="89"/>
-      <c r="P12" s="72" t="s">
+      <c r="B12" s="28"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="37"/>
+      <c r="F12" s="37"/>
+      <c r="G12" s="73"/>
+      <c r="H12" s="74"/>
+      <c r="I12" s="75"/>
+      <c r="J12" s="76"/>
+      <c r="K12" s="48"/>
+      <c r="L12" s="49"/>
+      <c r="N12" s="44"/>
+      <c r="O12" s="45"/>
+      <c r="P12" s="76" t="s">
         <v>20</v>
       </c>
-      <c r="Q12" s="73"/>
-      <c r="R12" s="74"/>
+      <c r="Q12" s="48"/>
+      <c r="R12" s="49"/>
     </row>
     <row r="13" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="28"/>
-      <c r="B13" s="30"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="39"/>
-      <c r="F13" s="39"/>
-      <c r="G13" s="69"/>
-      <c r="H13" s="70"/>
-      <c r="I13" s="71"/>
-      <c r="J13" s="72"/>
-      <c r="K13" s="73"/>
-      <c r="L13" s="74"/>
-      <c r="N13" s="88"/>
-      <c r="O13" s="89"/>
-      <c r="P13" s="72" t="s">
+      <c r="A13" s="107"/>
+      <c r="B13" s="29"/>
+      <c r="D13" s="27"/>
+      <c r="E13" s="37"/>
+      <c r="F13" s="37"/>
+      <c r="G13" s="73"/>
+      <c r="H13" s="74"/>
+      <c r="I13" s="75"/>
+      <c r="J13" s="76"/>
+      <c r="K13" s="48"/>
+      <c r="L13" s="49"/>
+      <c r="N13" s="44"/>
+      <c r="O13" s="45"/>
+      <c r="P13" s="76" t="s">
         <v>20</v>
       </c>
-      <c r="Q13" s="73"/>
-      <c r="R13" s="74"/>
+      <c r="Q13" s="48"/>
+      <c r="R13" s="49"/>
     </row>
     <row r="14" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="28" t="s">
+      <c r="A14" s="107" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="29"/>
-      <c r="D14" s="28"/>
-      <c r="E14" s="39"/>
-      <c r="F14" s="39"/>
-      <c r="G14" s="69"/>
-      <c r="H14" s="70"/>
-      <c r="I14" s="71"/>
-      <c r="J14" s="72"/>
-      <c r="K14" s="73"/>
-      <c r="L14" s="74"/>
+      <c r="B14" s="28"/>
+      <c r="D14" s="27"/>
+      <c r="E14" s="37"/>
+      <c r="F14" s="37"/>
+      <c r="G14" s="73"/>
+      <c r="H14" s="74"/>
+      <c r="I14" s="75"/>
+      <c r="J14" s="76"/>
+      <c r="K14" s="48"/>
+      <c r="L14" s="49"/>
       <c r="M14" t="s">
         <v>20</v>
       </c>
-      <c r="N14" s="88"/>
-      <c r="O14" s="89"/>
-      <c r="P14" s="72" t="s">
+      <c r="N14" s="44"/>
+      <c r="O14" s="45"/>
+      <c r="P14" s="76" t="s">
         <v>20</v>
       </c>
-      <c r="Q14" s="73"/>
-      <c r="R14" s="74"/>
+      <c r="Q14" s="48"/>
+      <c r="R14" s="49"/>
     </row>
     <row r="15" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="28" t="s">
+      <c r="A15" s="107" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="29"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="39"/>
-      <c r="F15" s="39"/>
-      <c r="G15" s="69"/>
-      <c r="H15" s="70"/>
-      <c r="I15" s="71"/>
-      <c r="J15" s="72"/>
-      <c r="K15" s="73"/>
-      <c r="L15" s="74"/>
+      <c r="B15" s="28"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="37"/>
+      <c r="F15" s="37"/>
+      <c r="G15" s="73"/>
+      <c r="H15" s="74"/>
+      <c r="I15" s="75"/>
+      <c r="J15" s="76"/>
+      <c r="K15" s="48"/>
+      <c r="L15" s="49"/>
       <c r="M15" t="s">
         <v>20</v>
       </c>
-      <c r="N15" s="88"/>
-      <c r="O15" s="89"/>
-      <c r="P15" s="72" t="s">
+      <c r="N15" s="44"/>
+      <c r="O15" s="45"/>
+      <c r="P15" s="76" t="s">
         <v>20</v>
       </c>
-      <c r="Q15" s="73"/>
-      <c r="R15" s="74"/>
+      <c r="Q15" s="48"/>
+      <c r="R15" s="49"/>
     </row>
     <row r="16" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="28"/>
-      <c r="B16" s="29"/>
-      <c r="D16" s="28"/>
-      <c r="E16" s="39"/>
-      <c r="F16" s="39"/>
-      <c r="G16" s="69"/>
-      <c r="H16" s="70"/>
-      <c r="I16" s="71"/>
-      <c r="J16" s="72"/>
-      <c r="K16" s="73"/>
-      <c r="L16" s="74"/>
-      <c r="N16" s="88"/>
-      <c r="O16" s="89"/>
-      <c r="P16" s="72" t="s">
+      <c r="A16" s="107"/>
+      <c r="B16" s="28"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="37"/>
+      <c r="F16" s="37"/>
+      <c r="G16" s="73"/>
+      <c r="H16" s="74"/>
+      <c r="I16" s="75"/>
+      <c r="J16" s="76"/>
+      <c r="K16" s="48"/>
+      <c r="L16" s="49"/>
+      <c r="N16" s="44"/>
+      <c r="O16" s="45"/>
+      <c r="P16" s="76" t="s">
         <v>20</v>
       </c>
-      <c r="Q16" s="73"/>
-      <c r="R16" s="74"/>
+      <c r="Q16" s="48"/>
+      <c r="R16" s="49"/>
     </row>
     <row r="17" spans="1:18" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="28"/>
-      <c r="B17" s="29"/>
-      <c r="D17" s="28"/>
-      <c r="E17" s="39"/>
-      <c r="F17" s="39"/>
-      <c r="G17" s="69"/>
-      <c r="H17" s="70"/>
-      <c r="I17" s="71"/>
-      <c r="J17" s="72"/>
-      <c r="K17" s="73"/>
-      <c r="L17" s="74"/>
-      <c r="N17" s="96"/>
-      <c r="O17" s="97"/>
-      <c r="P17" s="98" t="s">
+      <c r="A17" s="107"/>
+      <c r="B17" s="28"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="37"/>
+      <c r="F17" s="37"/>
+      <c r="G17" s="73"/>
+      <c r="H17" s="74"/>
+      <c r="I17" s="75"/>
+      <c r="J17" s="76"/>
+      <c r="K17" s="48"/>
+      <c r="L17" s="49"/>
+      <c r="N17" s="50"/>
+      <c r="O17" s="51"/>
+      <c r="P17" s="77" t="s">
         <v>20</v>
       </c>
-      <c r="Q17" s="99"/>
-      <c r="R17" s="100"/>
+      <c r="Q17" s="54"/>
+      <c r="R17" s="55"/>
     </row>
     <row r="18" spans="1:18" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="31"/>
-      <c r="B18" s="32"/>
-      <c r="D18" s="28"/>
-      <c r="E18" s="39"/>
-      <c r="F18" s="39"/>
-      <c r="G18" s="69"/>
-      <c r="H18" s="70"/>
-      <c r="I18" s="71"/>
-      <c r="J18" s="72"/>
-      <c r="K18" s="73"/>
-      <c r="L18" s="74"/>
+      <c r="A18" s="108"/>
+      <c r="B18" s="30"/>
+      <c r="D18" s="27"/>
+      <c r="E18" s="37"/>
+      <c r="F18" s="37"/>
+      <c r="G18" s="73"/>
+      <c r="H18" s="74"/>
+      <c r="I18" s="75"/>
+      <c r="J18" s="76"/>
+      <c r="K18" s="48"/>
+      <c r="L18" s="49"/>
     </row>
     <row r="19" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="90" t="s">
+      <c r="A19" s="62" t="s">
         <v>21</v>
       </c>
-      <c r="B19" s="91"/>
-      <c r="D19" s="92" t="s">
+      <c r="B19" s="63"/>
+      <c r="D19" s="64" t="s">
         <v>22</v>
       </c>
-      <c r="E19" s="93"/>
-      <c r="F19" s="93"/>
-      <c r="G19" s="93"/>
-      <c r="H19" s="93"/>
-      <c r="I19" s="93"/>
-      <c r="J19" s="93"/>
-      <c r="K19" s="93"/>
-      <c r="L19" s="94"/>
-      <c r="N19" s="92" t="s">
+      <c r="E19" s="65"/>
+      <c r="F19" s="65"/>
+      <c r="G19" s="65"/>
+      <c r="H19" s="65"/>
+      <c r="I19" s="65"/>
+      <c r="J19" s="65"/>
+      <c r="K19" s="65"/>
+      <c r="L19" s="66"/>
+      <c r="N19" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="O19" s="93"/>
-      <c r="P19" s="93"/>
-      <c r="Q19" s="93"/>
-      <c r="R19" s="94"/>
+      <c r="O19" s="65"/>
+      <c r="P19" s="65"/>
+      <c r="Q19" s="65"/>
+      <c r="R19" s="66"/>
     </row>
     <row r="20" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="19" t="s">
@@ -2133,370 +2140,370 @@
       <c r="B20" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D20" s="95" t="s">
+      <c r="D20" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="E20" s="86"/>
-      <c r="F20" s="84" t="s">
+      <c r="E20" s="68"/>
+      <c r="F20" s="69" t="s">
         <v>17</v>
       </c>
-      <c r="G20" s="85"/>
-      <c r="H20" s="85"/>
-      <c r="I20" s="85"/>
-      <c r="J20" s="85"/>
-      <c r="K20" s="85"/>
+      <c r="G20" s="70"/>
+      <c r="H20" s="70"/>
+      <c r="I20" s="70"/>
+      <c r="J20" s="70"/>
+      <c r="K20" s="70"/>
       <c r="L20" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="N20" s="75"/>
-      <c r="O20" s="65"/>
-      <c r="P20" s="65"/>
-      <c r="Q20" s="65"/>
-      <c r="R20" s="66"/>
+      <c r="N20" s="58"/>
+      <c r="O20" s="71"/>
+      <c r="P20" s="71"/>
+      <c r="Q20" s="71"/>
+      <c r="R20" s="72"/>
     </row>
     <row r="21" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="28"/>
-      <c r="B21" s="29"/>
-      <c r="D21" s="75"/>
-      <c r="E21" s="76"/>
-      <c r="F21" s="103"/>
-      <c r="G21" s="104"/>
-      <c r="H21" s="104"/>
-      <c r="I21" s="104"/>
-      <c r="J21" s="104"/>
-      <c r="K21" s="104"/>
-      <c r="L21" s="40"/>
-      <c r="N21" s="88"/>
-      <c r="O21" s="73"/>
-      <c r="P21" s="73"/>
-      <c r="Q21" s="73"/>
-      <c r="R21" s="74"/>
+      <c r="A21" s="107"/>
+      <c r="B21" s="28"/>
+      <c r="D21" s="58"/>
+      <c r="E21" s="59"/>
+      <c r="F21" s="60"/>
+      <c r="G21" s="61"/>
+      <c r="H21" s="61"/>
+      <c r="I21" s="61"/>
+      <c r="J21" s="61"/>
+      <c r="K21" s="61"/>
+      <c r="L21" s="38"/>
+      <c r="N21" s="44"/>
+      <c r="O21" s="48"/>
+      <c r="P21" s="48"/>
+      <c r="Q21" s="48"/>
+      <c r="R21" s="49"/>
     </row>
     <row r="22" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="28"/>
-      <c r="B22" s="29"/>
-      <c r="D22" s="88"/>
-      <c r="E22" s="89"/>
-      <c r="F22" s="101"/>
-      <c r="G22" s="102"/>
-      <c r="H22" s="102"/>
-      <c r="I22" s="102"/>
-      <c r="J22" s="102"/>
-      <c r="K22" s="102"/>
-      <c r="L22" s="41"/>
-      <c r="N22" s="88"/>
-      <c r="O22" s="73"/>
-      <c r="P22" s="73"/>
-      <c r="Q22" s="73"/>
-      <c r="R22" s="74"/>
+      <c r="A22" s="107"/>
+      <c r="B22" s="28"/>
+      <c r="D22" s="44"/>
+      <c r="E22" s="45"/>
+      <c r="F22" s="46"/>
+      <c r="G22" s="47"/>
+      <c r="H22" s="47"/>
+      <c r="I22" s="47"/>
+      <c r="J22" s="47"/>
+      <c r="K22" s="47"/>
+      <c r="L22" s="39"/>
+      <c r="N22" s="44"/>
+      <c r="O22" s="48"/>
+      <c r="P22" s="48"/>
+      <c r="Q22" s="48"/>
+      <c r="R22" s="49"/>
     </row>
     <row r="23" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="28"/>
-      <c r="B23" s="29"/>
-      <c r="D23" s="88"/>
-      <c r="E23" s="89"/>
-      <c r="F23" s="101"/>
-      <c r="G23" s="102"/>
-      <c r="H23" s="102"/>
-      <c r="I23" s="102"/>
-      <c r="J23" s="102"/>
-      <c r="K23" s="102"/>
-      <c r="L23" s="41"/>
-      <c r="N23" s="88"/>
-      <c r="O23" s="73"/>
-      <c r="P23" s="73"/>
-      <c r="Q23" s="73"/>
-      <c r="R23" s="74"/>
+      <c r="A23" s="107"/>
+      <c r="B23" s="28"/>
+      <c r="D23" s="44"/>
+      <c r="E23" s="45"/>
+      <c r="F23" s="46"/>
+      <c r="G23" s="47"/>
+      <c r="H23" s="47"/>
+      <c r="I23" s="47"/>
+      <c r="J23" s="47"/>
+      <c r="K23" s="47"/>
+      <c r="L23" s="39"/>
+      <c r="N23" s="44"/>
+      <c r="O23" s="48"/>
+      <c r="P23" s="48"/>
+      <c r="Q23" s="48"/>
+      <c r="R23" s="49"/>
     </row>
     <row r="24" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="28"/>
-      <c r="B24" s="29"/>
-      <c r="D24" s="88"/>
-      <c r="E24" s="89"/>
-      <c r="F24" s="101"/>
-      <c r="G24" s="102"/>
-      <c r="H24" s="102"/>
-      <c r="I24" s="102"/>
-      <c r="J24" s="102"/>
-      <c r="K24" s="102"/>
-      <c r="L24" s="41"/>
-      <c r="N24" s="88"/>
-      <c r="O24" s="73"/>
-      <c r="P24" s="73"/>
-      <c r="Q24" s="73"/>
-      <c r="R24" s="74"/>
+      <c r="A24" s="107"/>
+      <c r="B24" s="28"/>
+      <c r="D24" s="44"/>
+      <c r="E24" s="45"/>
+      <c r="F24" s="46"/>
+      <c r="G24" s="47"/>
+      <c r="H24" s="47"/>
+      <c r="I24" s="47"/>
+      <c r="J24" s="47"/>
+      <c r="K24" s="47"/>
+      <c r="L24" s="39"/>
+      <c r="N24" s="44"/>
+      <c r="O24" s="48"/>
+      <c r="P24" s="48"/>
+      <c r="Q24" s="48"/>
+      <c r="R24" s="49"/>
     </row>
     <row r="25" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="28"/>
-      <c r="B25" s="29"/>
-      <c r="D25" s="88"/>
-      <c r="E25" s="89"/>
-      <c r="F25" s="101"/>
-      <c r="G25" s="102"/>
-      <c r="H25" s="102"/>
-      <c r="I25" s="102"/>
-      <c r="J25" s="102"/>
-      <c r="K25" s="102"/>
-      <c r="L25" s="41"/>
-      <c r="N25" s="88"/>
-      <c r="O25" s="73"/>
-      <c r="P25" s="73"/>
-      <c r="Q25" s="73"/>
-      <c r="R25" s="74"/>
+      <c r="A25" s="107"/>
+      <c r="B25" s="28"/>
+      <c r="D25" s="44"/>
+      <c r="E25" s="45"/>
+      <c r="F25" s="46"/>
+      <c r="G25" s="47"/>
+      <c r="H25" s="47"/>
+      <c r="I25" s="47"/>
+      <c r="J25" s="47"/>
+      <c r="K25" s="47"/>
+      <c r="L25" s="39"/>
+      <c r="N25" s="44"/>
+      <c r="O25" s="48"/>
+      <c r="P25" s="48"/>
+      <c r="Q25" s="48"/>
+      <c r="R25" s="49"/>
     </row>
     <row r="26" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="28"/>
-      <c r="B26" s="29"/>
-      <c r="D26" s="88"/>
-      <c r="E26" s="89"/>
-      <c r="F26" s="101"/>
-      <c r="G26" s="102"/>
-      <c r="H26" s="102"/>
-      <c r="I26" s="102"/>
-      <c r="J26" s="102"/>
-      <c r="K26" s="102"/>
-      <c r="L26" s="41"/>
-      <c r="N26" s="88"/>
-      <c r="O26" s="73"/>
-      <c r="P26" s="73"/>
-      <c r="Q26" s="73"/>
-      <c r="R26" s="74"/>
+      <c r="A26" s="107"/>
+      <c r="B26" s="28"/>
+      <c r="D26" s="44"/>
+      <c r="E26" s="45"/>
+      <c r="F26" s="46"/>
+      <c r="G26" s="47"/>
+      <c r="H26" s="47"/>
+      <c r="I26" s="47"/>
+      <c r="J26" s="47"/>
+      <c r="K26" s="47"/>
+      <c r="L26" s="39"/>
+      <c r="N26" s="44"/>
+      <c r="O26" s="48"/>
+      <c r="P26" s="48"/>
+      <c r="Q26" s="48"/>
+      <c r="R26" s="49"/>
     </row>
     <row r="27" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="28"/>
-      <c r="B27" s="29"/>
-      <c r="D27" s="88"/>
-      <c r="E27" s="89"/>
-      <c r="F27" s="101"/>
-      <c r="G27" s="102"/>
-      <c r="H27" s="102"/>
-      <c r="I27" s="102"/>
-      <c r="J27" s="102"/>
-      <c r="K27" s="102"/>
-      <c r="L27" s="41"/>
-      <c r="N27" s="88"/>
-      <c r="O27" s="73"/>
-      <c r="P27" s="73"/>
-      <c r="Q27" s="73"/>
-      <c r="R27" s="74"/>
+      <c r="A27" s="107"/>
+      <c r="B27" s="28"/>
+      <c r="D27" s="44"/>
+      <c r="E27" s="45"/>
+      <c r="F27" s="46"/>
+      <c r="G27" s="47"/>
+      <c r="H27" s="47"/>
+      <c r="I27" s="47"/>
+      <c r="J27" s="47"/>
+      <c r="K27" s="47"/>
+      <c r="L27" s="39"/>
+      <c r="N27" s="44"/>
+      <c r="O27" s="48"/>
+      <c r="P27" s="48"/>
+      <c r="Q27" s="48"/>
+      <c r="R27" s="49"/>
     </row>
     <row r="28" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="28"/>
-      <c r="B28" s="29"/>
-      <c r="D28" s="88"/>
-      <c r="E28" s="89"/>
-      <c r="F28" s="101"/>
-      <c r="G28" s="102"/>
-      <c r="H28" s="102"/>
-      <c r="I28" s="102"/>
-      <c r="J28" s="102"/>
-      <c r="K28" s="102"/>
-      <c r="L28" s="41"/>
-      <c r="N28" s="88"/>
-      <c r="O28" s="73"/>
-      <c r="P28" s="73"/>
-      <c r="Q28" s="73"/>
-      <c r="R28" s="74"/>
+      <c r="A28" s="107"/>
+      <c r="B28" s="28"/>
+      <c r="D28" s="44"/>
+      <c r="E28" s="45"/>
+      <c r="F28" s="46"/>
+      <c r="G28" s="47"/>
+      <c r="H28" s="47"/>
+      <c r="I28" s="47"/>
+      <c r="J28" s="47"/>
+      <c r="K28" s="47"/>
+      <c r="L28" s="39"/>
+      <c r="N28" s="44"/>
+      <c r="O28" s="48"/>
+      <c r="P28" s="48"/>
+      <c r="Q28" s="48"/>
+      <c r="R28" s="49"/>
     </row>
     <row r="29" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="28"/>
-      <c r="B29" s="29"/>
-      <c r="D29" s="88"/>
-      <c r="E29" s="89"/>
-      <c r="F29" s="101"/>
-      <c r="G29" s="102"/>
-      <c r="H29" s="102"/>
-      <c r="I29" s="102"/>
-      <c r="J29" s="102"/>
-      <c r="K29" s="102"/>
-      <c r="L29" s="41"/>
-      <c r="N29" s="88"/>
-      <c r="O29" s="73"/>
-      <c r="P29" s="73"/>
-      <c r="Q29" s="73"/>
-      <c r="R29" s="74"/>
+      <c r="A29" s="107"/>
+      <c r="B29" s="28"/>
+      <c r="D29" s="44"/>
+      <c r="E29" s="45"/>
+      <c r="F29" s="46"/>
+      <c r="G29" s="47"/>
+      <c r="H29" s="47"/>
+      <c r="I29" s="47"/>
+      <c r="J29" s="47"/>
+      <c r="K29" s="47"/>
+      <c r="L29" s="39"/>
+      <c r="N29" s="44"/>
+      <c r="O29" s="48"/>
+      <c r="P29" s="48"/>
+      <c r="Q29" s="48"/>
+      <c r="R29" s="49"/>
     </row>
     <row r="30" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="28"/>
-      <c r="B30" s="29"/>
-      <c r="D30" s="88"/>
-      <c r="E30" s="89"/>
-      <c r="F30" s="101"/>
-      <c r="G30" s="102"/>
-      <c r="H30" s="102"/>
-      <c r="I30" s="102"/>
-      <c r="J30" s="102"/>
-      <c r="K30" s="102"/>
-      <c r="L30" s="41"/>
-      <c r="N30" s="88"/>
-      <c r="O30" s="73"/>
-      <c r="P30" s="73"/>
-      <c r="Q30" s="73"/>
-      <c r="R30" s="74"/>
+      <c r="A30" s="107"/>
+      <c r="B30" s="28"/>
+      <c r="D30" s="44"/>
+      <c r="E30" s="45"/>
+      <c r="F30" s="46"/>
+      <c r="G30" s="47"/>
+      <c r="H30" s="47"/>
+      <c r="I30" s="47"/>
+      <c r="J30" s="47"/>
+      <c r="K30" s="47"/>
+      <c r="L30" s="39"/>
+      <c r="N30" s="44"/>
+      <c r="O30" s="48"/>
+      <c r="P30" s="48"/>
+      <c r="Q30" s="48"/>
+      <c r="R30" s="49"/>
     </row>
     <row r="31" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="28"/>
-      <c r="B31" s="29"/>
-      <c r="D31" s="88"/>
-      <c r="E31" s="89"/>
-      <c r="F31" s="101"/>
-      <c r="G31" s="102"/>
-      <c r="H31" s="102"/>
-      <c r="I31" s="102"/>
-      <c r="J31" s="102"/>
-      <c r="K31" s="102"/>
-      <c r="L31" s="41"/>
-      <c r="N31" s="88"/>
-      <c r="O31" s="73"/>
-      <c r="P31" s="73"/>
-      <c r="Q31" s="73"/>
-      <c r="R31" s="74"/>
+      <c r="A31" s="107"/>
+      <c r="B31" s="28"/>
+      <c r="D31" s="44"/>
+      <c r="E31" s="45"/>
+      <c r="F31" s="46"/>
+      <c r="G31" s="47"/>
+      <c r="H31" s="47"/>
+      <c r="I31" s="47"/>
+      <c r="J31" s="47"/>
+      <c r="K31" s="47"/>
+      <c r="L31" s="39"/>
+      <c r="N31" s="44"/>
+      <c r="O31" s="48"/>
+      <c r="P31" s="48"/>
+      <c r="Q31" s="48"/>
+      <c r="R31" s="49"/>
     </row>
     <row r="32" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="28"/>
-      <c r="B32" s="29"/>
-      <c r="D32" s="88"/>
-      <c r="E32" s="89"/>
-      <c r="F32" s="101"/>
-      <c r="G32" s="102"/>
-      <c r="H32" s="102"/>
-      <c r="I32" s="102"/>
-      <c r="J32" s="102"/>
-      <c r="K32" s="102"/>
-      <c r="L32" s="41"/>
-      <c r="N32" s="88"/>
-      <c r="O32" s="73"/>
-      <c r="P32" s="73"/>
-      <c r="Q32" s="73"/>
-      <c r="R32" s="74"/>
+      <c r="A32" s="107"/>
+      <c r="B32" s="28"/>
+      <c r="D32" s="44"/>
+      <c r="E32" s="45"/>
+      <c r="F32" s="46"/>
+      <c r="G32" s="47"/>
+      <c r="H32" s="47"/>
+      <c r="I32" s="47"/>
+      <c r="J32" s="47"/>
+      <c r="K32" s="47"/>
+      <c r="L32" s="39"/>
+      <c r="N32" s="44"/>
+      <c r="O32" s="48"/>
+      <c r="P32" s="48"/>
+      <c r="Q32" s="48"/>
+      <c r="R32" s="49"/>
     </row>
     <row r="33" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="28"/>
-      <c r="B33" s="29"/>
-      <c r="D33" s="88"/>
-      <c r="E33" s="89"/>
-      <c r="F33" s="101"/>
-      <c r="G33" s="102"/>
-      <c r="H33" s="102"/>
-      <c r="I33" s="102"/>
-      <c r="J33" s="102"/>
-      <c r="K33" s="102"/>
-      <c r="L33" s="41"/>
-      <c r="N33" s="88"/>
-      <c r="O33" s="73"/>
-      <c r="P33" s="73"/>
-      <c r="Q33" s="73"/>
-      <c r="R33" s="74"/>
+      <c r="A33" s="107"/>
+      <c r="B33" s="28"/>
+      <c r="D33" s="44"/>
+      <c r="E33" s="45"/>
+      <c r="F33" s="46"/>
+      <c r="G33" s="47"/>
+      <c r="H33" s="47"/>
+      <c r="I33" s="47"/>
+      <c r="J33" s="47"/>
+      <c r="K33" s="47"/>
+      <c r="L33" s="39"/>
+      <c r="N33" s="44"/>
+      <c r="O33" s="48"/>
+      <c r="P33" s="48"/>
+      <c r="Q33" s="48"/>
+      <c r="R33" s="49"/>
     </row>
     <row r="34" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="28"/>
-      <c r="B34" s="29"/>
-      <c r="D34" s="88"/>
-      <c r="E34" s="89"/>
-      <c r="F34" s="101"/>
-      <c r="G34" s="102"/>
-      <c r="H34" s="102"/>
-      <c r="I34" s="102"/>
-      <c r="J34" s="102"/>
-      <c r="K34" s="102"/>
-      <c r="L34" s="41"/>
-      <c r="N34" s="88"/>
-      <c r="O34" s="73"/>
-      <c r="P34" s="73"/>
-      <c r="Q34" s="73"/>
-      <c r="R34" s="74"/>
+      <c r="A34" s="107"/>
+      <c r="B34" s="28"/>
+      <c r="D34" s="44"/>
+      <c r="E34" s="45"/>
+      <c r="F34" s="46"/>
+      <c r="G34" s="47"/>
+      <c r="H34" s="47"/>
+      <c r="I34" s="47"/>
+      <c r="J34" s="47"/>
+      <c r="K34" s="47"/>
+      <c r="L34" s="39"/>
+      <c r="N34" s="44"/>
+      <c r="O34" s="48"/>
+      <c r="P34" s="48"/>
+      <c r="Q34" s="48"/>
+      <c r="R34" s="49"/>
     </row>
     <row r="35" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="28"/>
-      <c r="B35" s="29"/>
-      <c r="D35" s="88"/>
-      <c r="E35" s="89"/>
-      <c r="F35" s="101"/>
-      <c r="G35" s="102"/>
-      <c r="H35" s="102"/>
-      <c r="I35" s="102"/>
-      <c r="J35" s="102"/>
-      <c r="K35" s="102"/>
-      <c r="L35" s="41"/>
-      <c r="N35" s="88"/>
-      <c r="O35" s="73"/>
-      <c r="P35" s="73"/>
-      <c r="Q35" s="73"/>
-      <c r="R35" s="74"/>
+      <c r="A35" s="107"/>
+      <c r="B35" s="28"/>
+      <c r="D35" s="44"/>
+      <c r="E35" s="45"/>
+      <c r="F35" s="46"/>
+      <c r="G35" s="47"/>
+      <c r="H35" s="47"/>
+      <c r="I35" s="47"/>
+      <c r="J35" s="47"/>
+      <c r="K35" s="47"/>
+      <c r="L35" s="39"/>
+      <c r="N35" s="44"/>
+      <c r="O35" s="48"/>
+      <c r="P35" s="48"/>
+      <c r="Q35" s="48"/>
+      <c r="R35" s="49"/>
     </row>
     <row r="36" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="28"/>
-      <c r="B36" s="29"/>
-      <c r="D36" s="88"/>
-      <c r="E36" s="89"/>
-      <c r="F36" s="101"/>
-      <c r="G36" s="102"/>
-      <c r="H36" s="102"/>
-      <c r="I36" s="102"/>
-      <c r="J36" s="102"/>
-      <c r="K36" s="102"/>
-      <c r="L36" s="41"/>
-      <c r="N36" s="88"/>
-      <c r="O36" s="73"/>
-      <c r="P36" s="73"/>
-      <c r="Q36" s="73"/>
-      <c r="R36" s="74"/>
+      <c r="A36" s="107"/>
+      <c r="B36" s="28"/>
+      <c r="D36" s="44"/>
+      <c r="E36" s="45"/>
+      <c r="F36" s="46"/>
+      <c r="G36" s="47"/>
+      <c r="H36" s="47"/>
+      <c r="I36" s="47"/>
+      <c r="J36" s="47"/>
+      <c r="K36" s="47"/>
+      <c r="L36" s="39"/>
+      <c r="N36" s="44"/>
+      <c r="O36" s="48"/>
+      <c r="P36" s="48"/>
+      <c r="Q36" s="48"/>
+      <c r="R36" s="49"/>
     </row>
     <row r="37" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="28"/>
-      <c r="B37" s="29"/>
-      <c r="D37" s="88"/>
-      <c r="E37" s="89"/>
-      <c r="F37" s="101"/>
-      <c r="G37" s="102"/>
-      <c r="H37" s="102"/>
-      <c r="I37" s="102"/>
-      <c r="J37" s="102"/>
-      <c r="K37" s="102"/>
-      <c r="L37" s="41"/>
-      <c r="N37" s="88"/>
-      <c r="O37" s="73"/>
-      <c r="P37" s="73"/>
-      <c r="Q37" s="73"/>
-      <c r="R37" s="74"/>
+      <c r="A37" s="107"/>
+      <c r="B37" s="28"/>
+      <c r="D37" s="44"/>
+      <c r="E37" s="45"/>
+      <c r="F37" s="46"/>
+      <c r="G37" s="47"/>
+      <c r="H37" s="47"/>
+      <c r="I37" s="47"/>
+      <c r="J37" s="47"/>
+      <c r="K37" s="47"/>
+      <c r="L37" s="39"/>
+      <c r="N37" s="44"/>
+      <c r="O37" s="48"/>
+      <c r="P37" s="48"/>
+      <c r="Q37" s="48"/>
+      <c r="R37" s="49"/>
     </row>
     <row r="38" spans="1:18" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="31"/>
-      <c r="B38" s="32"/>
-      <c r="D38" s="88"/>
-      <c r="E38" s="89"/>
-      <c r="F38" s="101"/>
-      <c r="G38" s="102"/>
-      <c r="H38" s="102"/>
-      <c r="I38" s="102"/>
-      <c r="J38" s="102"/>
-      <c r="K38" s="102"/>
-      <c r="L38" s="41"/>
-      <c r="N38" s="88"/>
-      <c r="O38" s="73"/>
-      <c r="P38" s="73"/>
-      <c r="Q38" s="73"/>
-      <c r="R38" s="74"/>
+      <c r="A38" s="108"/>
+      <c r="B38" s="30"/>
+      <c r="D38" s="44"/>
+      <c r="E38" s="45"/>
+      <c r="F38" s="46"/>
+      <c r="G38" s="47"/>
+      <c r="H38" s="47"/>
+      <c r="I38" s="47"/>
+      <c r="J38" s="47"/>
+      <c r="K38" s="47"/>
+      <c r="L38" s="39"/>
+      <c r="N38" s="44"/>
+      <c r="O38" s="48"/>
+      <c r="P38" s="48"/>
+      <c r="Q38" s="48"/>
+      <c r="R38" s="49"/>
     </row>
     <row r="39" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="105" t="s">
+      <c r="A39" s="56" t="s">
         <v>26</v>
       </c>
-      <c r="B39" s="106"/>
-      <c r="D39" s="88"/>
-      <c r="E39" s="89"/>
-      <c r="F39" s="101"/>
-      <c r="G39" s="102"/>
-      <c r="H39" s="102"/>
-      <c r="I39" s="102"/>
-      <c r="J39" s="102"/>
-      <c r="K39" s="102"/>
-      <c r="L39" s="41"/>
-      <c r="N39" s="88"/>
-      <c r="O39" s="73"/>
-      <c r="P39" s="73"/>
-      <c r="Q39" s="73"/>
-      <c r="R39" s="74"/>
+      <c r="B39" s="57"/>
+      <c r="D39" s="44"/>
+      <c r="E39" s="45"/>
+      <c r="F39" s="46"/>
+      <c r="G39" s="47"/>
+      <c r="H39" s="47"/>
+      <c r="I39" s="47"/>
+      <c r="J39" s="47"/>
+      <c r="K39" s="47"/>
+      <c r="L39" s="39"/>
+      <c r="N39" s="44"/>
+      <c r="O39" s="48"/>
+      <c r="P39" s="48"/>
+      <c r="Q39" s="48"/>
+      <c r="R39" s="49"/>
     </row>
     <row r="40" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="22" t="s">
@@ -2505,349 +2512,270 @@
       <c r="B40" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="D40" s="88"/>
-      <c r="E40" s="89"/>
-      <c r="F40" s="101"/>
-      <c r="G40" s="102"/>
-      <c r="H40" s="102"/>
-      <c r="I40" s="102"/>
-      <c r="J40" s="102"/>
-      <c r="K40" s="102"/>
-      <c r="L40" s="41"/>
-      <c r="N40" s="88"/>
-      <c r="O40" s="73"/>
-      <c r="P40" s="73"/>
-      <c r="Q40" s="73"/>
-      <c r="R40" s="74"/>
+      <c r="D40" s="44"/>
+      <c r="E40" s="45"/>
+      <c r="F40" s="46"/>
+      <c r="G40" s="47"/>
+      <c r="H40" s="47"/>
+      <c r="I40" s="47"/>
+      <c r="J40" s="47"/>
+      <c r="K40" s="47"/>
+      <c r="L40" s="39"/>
+      <c r="N40" s="44"/>
+      <c r="O40" s="48"/>
+      <c r="P40" s="48"/>
+      <c r="Q40" s="48"/>
+      <c r="R40" s="49"/>
     </row>
     <row r="41" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="28"/>
-      <c r="B41" s="29"/>
-      <c r="D41" s="88"/>
-      <c r="E41" s="89"/>
-      <c r="F41" s="101"/>
-      <c r="G41" s="102"/>
-      <c r="H41" s="102"/>
-      <c r="I41" s="102"/>
-      <c r="J41" s="102"/>
-      <c r="K41" s="102"/>
-      <c r="L41" s="41"/>
-      <c r="N41" s="88"/>
-      <c r="O41" s="73"/>
-      <c r="P41" s="73"/>
-      <c r="Q41" s="73"/>
-      <c r="R41" s="74"/>
+      <c r="A41" s="107"/>
+      <c r="B41" s="28"/>
+      <c r="D41" s="44"/>
+      <c r="E41" s="45"/>
+      <c r="F41" s="46"/>
+      <c r="G41" s="47"/>
+      <c r="H41" s="47"/>
+      <c r="I41" s="47"/>
+      <c r="J41" s="47"/>
+      <c r="K41" s="47"/>
+      <c r="L41" s="39"/>
+      <c r="N41" s="44"/>
+      <c r="O41" s="48"/>
+      <c r="P41" s="48"/>
+      <c r="Q41" s="48"/>
+      <c r="R41" s="49"/>
     </row>
     <row r="42" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="28"/>
-      <c r="B42" s="29"/>
-      <c r="D42" s="88"/>
-      <c r="E42" s="89"/>
-      <c r="F42" s="101"/>
-      <c r="G42" s="102"/>
-      <c r="H42" s="102"/>
-      <c r="I42" s="102"/>
-      <c r="J42" s="102"/>
-      <c r="K42" s="102"/>
-      <c r="L42" s="41"/>
-      <c r="N42" s="88"/>
-      <c r="O42" s="73"/>
-      <c r="P42" s="73"/>
-      <c r="Q42" s="73"/>
-      <c r="R42" s="74"/>
+      <c r="A42" s="107"/>
+      <c r="B42" s="28"/>
+      <c r="D42" s="44"/>
+      <c r="E42" s="45"/>
+      <c r="F42" s="46"/>
+      <c r="G42" s="47"/>
+      <c r="H42" s="47"/>
+      <c r="I42" s="47"/>
+      <c r="J42" s="47"/>
+      <c r="K42" s="47"/>
+      <c r="L42" s="39"/>
+      <c r="N42" s="44"/>
+      <c r="O42" s="48"/>
+      <c r="P42" s="48"/>
+      <c r="Q42" s="48"/>
+      <c r="R42" s="49"/>
     </row>
     <row r="43" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="28"/>
-      <c r="B43" s="29"/>
-      <c r="D43" s="88"/>
-      <c r="E43" s="89"/>
-      <c r="F43" s="101"/>
-      <c r="G43" s="102"/>
-      <c r="H43" s="102"/>
-      <c r="I43" s="102"/>
-      <c r="J43" s="102"/>
-      <c r="K43" s="102"/>
-      <c r="L43" s="41"/>
-      <c r="N43" s="88"/>
-      <c r="O43" s="73"/>
-      <c r="P43" s="73"/>
-      <c r="Q43" s="73"/>
-      <c r="R43" s="74"/>
+      <c r="A43" s="107"/>
+      <c r="B43" s="28"/>
+      <c r="D43" s="44"/>
+      <c r="E43" s="45"/>
+      <c r="F43" s="46"/>
+      <c r="G43" s="47"/>
+      <c r="H43" s="47"/>
+      <c r="I43" s="47"/>
+      <c r="J43" s="47"/>
+      <c r="K43" s="47"/>
+      <c r="L43" s="39"/>
+      <c r="N43" s="44"/>
+      <c r="O43" s="48"/>
+      <c r="P43" s="48"/>
+      <c r="Q43" s="48"/>
+      <c r="R43" s="49"/>
     </row>
     <row r="44" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="28"/>
-      <c r="B44" s="29"/>
-      <c r="D44" s="88"/>
-      <c r="E44" s="89"/>
-      <c r="F44" s="101"/>
-      <c r="G44" s="102"/>
-      <c r="H44" s="102"/>
-      <c r="I44" s="102"/>
-      <c r="J44" s="102"/>
-      <c r="K44" s="102"/>
-      <c r="L44" s="41"/>
-      <c r="N44" s="88"/>
-      <c r="O44" s="73"/>
-      <c r="P44" s="73"/>
-      <c r="Q44" s="73"/>
-      <c r="R44" s="74"/>
+      <c r="A44" s="107"/>
+      <c r="B44" s="28"/>
+      <c r="D44" s="44"/>
+      <c r="E44" s="45"/>
+      <c r="F44" s="46"/>
+      <c r="G44" s="47"/>
+      <c r="H44" s="47"/>
+      <c r="I44" s="47"/>
+      <c r="J44" s="47"/>
+      <c r="K44" s="47"/>
+      <c r="L44" s="39"/>
+      <c r="N44" s="44"/>
+      <c r="O44" s="48"/>
+      <c r="P44" s="48"/>
+      <c r="Q44" s="48"/>
+      <c r="R44" s="49"/>
     </row>
     <row r="45" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="28"/>
-      <c r="B45" s="29"/>
-      <c r="D45" s="88"/>
-      <c r="E45" s="89"/>
-      <c r="F45" s="101"/>
-      <c r="G45" s="102"/>
-      <c r="H45" s="102"/>
-      <c r="I45" s="102"/>
-      <c r="J45" s="102"/>
-      <c r="K45" s="102"/>
-      <c r="L45" s="41"/>
-      <c r="N45" s="88"/>
-      <c r="O45" s="73"/>
-      <c r="P45" s="73"/>
-      <c r="Q45" s="73"/>
-      <c r="R45" s="74"/>
+      <c r="A45" s="107"/>
+      <c r="B45" s="28"/>
+      <c r="D45" s="44"/>
+      <c r="E45" s="45"/>
+      <c r="F45" s="46"/>
+      <c r="G45" s="47"/>
+      <c r="H45" s="47"/>
+      <c r="I45" s="47"/>
+      <c r="J45" s="47"/>
+      <c r="K45" s="47"/>
+      <c r="L45" s="39"/>
+      <c r="N45" s="44"/>
+      <c r="O45" s="48"/>
+      <c r="P45" s="48"/>
+      <c r="Q45" s="48"/>
+      <c r="R45" s="49"/>
     </row>
     <row r="46" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="28"/>
-      <c r="B46" s="29"/>
-      <c r="D46" s="88"/>
-      <c r="E46" s="89"/>
-      <c r="F46" s="101"/>
-      <c r="G46" s="102"/>
-      <c r="H46" s="102"/>
-      <c r="I46" s="102"/>
-      <c r="J46" s="102"/>
-      <c r="K46" s="102"/>
-      <c r="L46" s="41"/>
-      <c r="N46" s="88"/>
-      <c r="O46" s="73"/>
-      <c r="P46" s="73"/>
-      <c r="Q46" s="73"/>
-      <c r="R46" s="74"/>
+      <c r="A46" s="107"/>
+      <c r="B46" s="28"/>
+      <c r="D46" s="44"/>
+      <c r="E46" s="45"/>
+      <c r="F46" s="46"/>
+      <c r="G46" s="47"/>
+      <c r="H46" s="47"/>
+      <c r="I46" s="47"/>
+      <c r="J46" s="47"/>
+      <c r="K46" s="47"/>
+      <c r="L46" s="39"/>
+      <c r="N46" s="44"/>
+      <c r="O46" s="48"/>
+      <c r="P46" s="48"/>
+      <c r="Q46" s="48"/>
+      <c r="R46" s="49"/>
     </row>
     <row r="47" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="28"/>
-      <c r="B47" s="29"/>
-      <c r="D47" s="88"/>
-      <c r="E47" s="89"/>
-      <c r="F47" s="101"/>
-      <c r="G47" s="102"/>
-      <c r="H47" s="102"/>
-      <c r="I47" s="102"/>
-      <c r="J47" s="102"/>
-      <c r="K47" s="102"/>
-      <c r="L47" s="41"/>
-      <c r="N47" s="88"/>
-      <c r="O47" s="73"/>
-      <c r="P47" s="73"/>
-      <c r="Q47" s="73"/>
-      <c r="R47" s="74"/>
+      <c r="A47" s="107"/>
+      <c r="B47" s="28"/>
+      <c r="D47" s="44"/>
+      <c r="E47" s="45"/>
+      <c r="F47" s="46"/>
+      <c r="G47" s="47"/>
+      <c r="H47" s="47"/>
+      <c r="I47" s="47"/>
+      <c r="J47" s="47"/>
+      <c r="K47" s="47"/>
+      <c r="L47" s="39"/>
+      <c r="N47" s="44"/>
+      <c r="O47" s="48"/>
+      <c r="P47" s="48"/>
+      <c r="Q47" s="48"/>
+      <c r="R47" s="49"/>
     </row>
     <row r="48" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="28"/>
-      <c r="B48" s="29"/>
-      <c r="D48" s="88"/>
-      <c r="E48" s="89"/>
-      <c r="F48" s="101"/>
-      <c r="G48" s="102"/>
-      <c r="H48" s="102"/>
-      <c r="I48" s="102"/>
-      <c r="J48" s="102"/>
-      <c r="K48" s="102"/>
-      <c r="L48" s="41"/>
-      <c r="N48" s="88"/>
-      <c r="O48" s="73"/>
-      <c r="P48" s="73"/>
-      <c r="Q48" s="73"/>
-      <c r="R48" s="74"/>
+      <c r="A48" s="107"/>
+      <c r="B48" s="28"/>
+      <c r="D48" s="44"/>
+      <c r="E48" s="45"/>
+      <c r="F48" s="46"/>
+      <c r="G48" s="47"/>
+      <c r="H48" s="47"/>
+      <c r="I48" s="47"/>
+      <c r="J48" s="47"/>
+      <c r="K48" s="47"/>
+      <c r="L48" s="39"/>
+      <c r="N48" s="44"/>
+      <c r="O48" s="48"/>
+      <c r="P48" s="48"/>
+      <c r="Q48" s="48"/>
+      <c r="R48" s="49"/>
     </row>
     <row r="49" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="28"/>
-      <c r="B49" s="29"/>
-      <c r="D49" s="88"/>
-      <c r="E49" s="89"/>
-      <c r="F49" s="101"/>
-      <c r="G49" s="102"/>
-      <c r="H49" s="102"/>
-      <c r="I49" s="102"/>
-      <c r="J49" s="102"/>
-      <c r="K49" s="102"/>
-      <c r="L49" s="41"/>
-      <c r="N49" s="88"/>
-      <c r="O49" s="73"/>
-      <c r="P49" s="73"/>
-      <c r="Q49" s="73"/>
-      <c r="R49" s="74"/>
+      <c r="A49" s="107"/>
+      <c r="B49" s="28"/>
+      <c r="D49" s="44"/>
+      <c r="E49" s="45"/>
+      <c r="F49" s="46"/>
+      <c r="G49" s="47"/>
+      <c r="H49" s="47"/>
+      <c r="I49" s="47"/>
+      <c r="J49" s="47"/>
+      <c r="K49" s="47"/>
+      <c r="L49" s="39"/>
+      <c r="N49" s="44"/>
+      <c r="O49" s="48"/>
+      <c r="P49" s="48"/>
+      <c r="Q49" s="48"/>
+      <c r="R49" s="49"/>
     </row>
     <row r="50" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="28"/>
-      <c r="B50" s="29"/>
-      <c r="D50" s="88"/>
-      <c r="E50" s="89"/>
-      <c r="F50" s="101"/>
-      <c r="G50" s="102"/>
-      <c r="H50" s="102"/>
-      <c r="I50" s="102"/>
-      <c r="J50" s="102"/>
-      <c r="K50" s="102"/>
-      <c r="L50" s="42"/>
-      <c r="N50" s="88"/>
-      <c r="O50" s="73"/>
-      <c r="P50" s="73"/>
-      <c r="Q50" s="73"/>
-      <c r="R50" s="74"/>
+      <c r="A50" s="107"/>
+      <c r="B50" s="28"/>
+      <c r="D50" s="44"/>
+      <c r="E50" s="45"/>
+      <c r="F50" s="46"/>
+      <c r="G50" s="47"/>
+      <c r="H50" s="47"/>
+      <c r="I50" s="47"/>
+      <c r="J50" s="47"/>
+      <c r="K50" s="47"/>
+      <c r="L50" s="40"/>
+      <c r="N50" s="44"/>
+      <c r="O50" s="48"/>
+      <c r="P50" s="48"/>
+      <c r="Q50" s="48"/>
+      <c r="R50" s="49"/>
     </row>
     <row r="51" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="28"/>
-      <c r="B51" s="29"/>
-      <c r="D51" s="88"/>
-      <c r="E51" s="89"/>
-      <c r="F51" s="101"/>
-      <c r="G51" s="102"/>
-      <c r="H51" s="102"/>
-      <c r="I51" s="102"/>
-      <c r="J51" s="102"/>
-      <c r="K51" s="102"/>
-      <c r="L51" s="42"/>
-      <c r="N51" s="88"/>
-      <c r="O51" s="73"/>
-      <c r="P51" s="73"/>
-      <c r="Q51" s="73"/>
-      <c r="R51" s="74"/>
+      <c r="A51" s="107"/>
+      <c r="B51" s="28"/>
+      <c r="D51" s="44"/>
+      <c r="E51" s="45"/>
+      <c r="F51" s="46"/>
+      <c r="G51" s="47"/>
+      <c r="H51" s="47"/>
+      <c r="I51" s="47"/>
+      <c r="J51" s="47"/>
+      <c r="K51" s="47"/>
+      <c r="L51" s="40"/>
+      <c r="N51" s="44"/>
+      <c r="O51" s="48"/>
+      <c r="P51" s="48"/>
+      <c r="Q51" s="48"/>
+      <c r="R51" s="49"/>
     </row>
     <row r="52" spans="1:18" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="31"/>
-      <c r="B52" s="32"/>
-      <c r="D52" s="96"/>
-      <c r="E52" s="97"/>
-      <c r="F52" s="107"/>
-      <c r="G52" s="108"/>
-      <c r="H52" s="108"/>
-      <c r="I52" s="108"/>
-      <c r="J52" s="108"/>
-      <c r="K52" s="108"/>
-      <c r="L52" s="43"/>
-      <c r="N52" s="96"/>
-      <c r="O52" s="99"/>
-      <c r="P52" s="99"/>
-      <c r="Q52" s="99"/>
-      <c r="R52" s="100"/>
+      <c r="A52" s="108"/>
+      <c r="B52" s="30"/>
+      <c r="D52" s="50"/>
+      <c r="E52" s="51"/>
+      <c r="F52" s="52"/>
+      <c r="G52" s="53"/>
+      <c r="H52" s="53"/>
+      <c r="I52" s="53"/>
+      <c r="J52" s="53"/>
+      <c r="K52" s="53"/>
+      <c r="L52" s="41"/>
+      <c r="N52" s="50"/>
+      <c r="O52" s="54"/>
+      <c r="P52" s="54"/>
+      <c r="Q52" s="54"/>
+      <c r="R52" s="55"/>
     </row>
     <row r="53" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="155">
-    <mergeCell ref="D51:E51"/>
-    <mergeCell ref="F51:K51"/>
-    <mergeCell ref="N51:R51"/>
-    <mergeCell ref="D52:E52"/>
-    <mergeCell ref="F52:K52"/>
-    <mergeCell ref="D49:E49"/>
-    <mergeCell ref="F49:K49"/>
-    <mergeCell ref="N49:R49"/>
-    <mergeCell ref="D50:E50"/>
-    <mergeCell ref="F50:K50"/>
-    <mergeCell ref="N50:R50"/>
-    <mergeCell ref="N52:R52"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="F47:K47"/>
-    <mergeCell ref="N47:R47"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="F48:K48"/>
-    <mergeCell ref="N48:R48"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="F45:K45"/>
-    <mergeCell ref="N45:R45"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="F46:K46"/>
-    <mergeCell ref="N46:R46"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="F43:K43"/>
-    <mergeCell ref="N43:R43"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="F44:K44"/>
-    <mergeCell ref="N44:R44"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="F41:K41"/>
-    <mergeCell ref="N41:R41"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="F42:K42"/>
-    <mergeCell ref="N42:R42"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="F39:K39"/>
-    <mergeCell ref="N39:R39"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="F40:K40"/>
-    <mergeCell ref="N40:R40"/>
-    <mergeCell ref="D37:E37"/>
-    <mergeCell ref="F37:K37"/>
-    <mergeCell ref="N37:R37"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="F38:K38"/>
-    <mergeCell ref="N38:R38"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="F35:K35"/>
-    <mergeCell ref="N35:R35"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="F36:K36"/>
-    <mergeCell ref="N36:R36"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="F33:K33"/>
-    <mergeCell ref="N33:R33"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="F34:K34"/>
-    <mergeCell ref="N34:R34"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="F31:K31"/>
-    <mergeCell ref="N31:R31"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="F32:K32"/>
-    <mergeCell ref="N32:R32"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="F29:K29"/>
-    <mergeCell ref="N29:R29"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="F30:K30"/>
-    <mergeCell ref="N30:R30"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="F27:K27"/>
-    <mergeCell ref="N27:R27"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="F28:K28"/>
-    <mergeCell ref="N28:R28"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="F25:K25"/>
-    <mergeCell ref="N25:R25"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="F26:K26"/>
-    <mergeCell ref="N26:R26"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="F23:K23"/>
-    <mergeCell ref="N23:R23"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="F24:K24"/>
-    <mergeCell ref="N24:R24"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="F21:K21"/>
-    <mergeCell ref="N21:R21"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="F22:K22"/>
-    <mergeCell ref="N22:R22"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="D19:L19"/>
-    <mergeCell ref="N19:R19"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="F20:K20"/>
-    <mergeCell ref="N20:R20"/>
-    <mergeCell ref="G17:I17"/>
-    <mergeCell ref="J17:L17"/>
-    <mergeCell ref="N17:O17"/>
-    <mergeCell ref="P17:R17"/>
-    <mergeCell ref="G18:I18"/>
-    <mergeCell ref="J18:L18"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="G3:I3"/>
+    <mergeCell ref="J3:L3"/>
+    <mergeCell ref="M3:Q3"/>
+    <mergeCell ref="R3:R7"/>
+    <mergeCell ref="G4:I4"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="M4:Q4"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="J9:L9"/>
+    <mergeCell ref="N9:O9"/>
+    <mergeCell ref="G10:I10"/>
+    <mergeCell ref="J10:L10"/>
+    <mergeCell ref="N10:O10"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:L5"/>
+    <mergeCell ref="A6:B7"/>
+    <mergeCell ref="D6:L7"/>
+    <mergeCell ref="G8:I8"/>
+    <mergeCell ref="J8:L8"/>
+    <mergeCell ref="P10:R10"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J11:L11"/>
+    <mergeCell ref="N11:O11"/>
+    <mergeCell ref="P11:R11"/>
+    <mergeCell ref="G12:I12"/>
+    <mergeCell ref="J12:L12"/>
+    <mergeCell ref="N12:O12"/>
+    <mergeCell ref="P12:R12"/>
     <mergeCell ref="G15:I15"/>
     <mergeCell ref="J15:L15"/>
     <mergeCell ref="N15:O15"/>
@@ -2864,36 +2792,115 @@
     <mergeCell ref="J14:L14"/>
     <mergeCell ref="N14:O14"/>
     <mergeCell ref="P14:R14"/>
-    <mergeCell ref="P10:R10"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="J11:L11"/>
-    <mergeCell ref="N11:O11"/>
-    <mergeCell ref="P11:R11"/>
-    <mergeCell ref="G12:I12"/>
-    <mergeCell ref="J12:L12"/>
-    <mergeCell ref="N12:O12"/>
-    <mergeCell ref="P12:R12"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="J9:L9"/>
-    <mergeCell ref="N9:O9"/>
-    <mergeCell ref="G10:I10"/>
-    <mergeCell ref="J10:L10"/>
-    <mergeCell ref="N10:O10"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:L5"/>
-    <mergeCell ref="A6:B7"/>
-    <mergeCell ref="D6:L7"/>
-    <mergeCell ref="G8:I8"/>
-    <mergeCell ref="J8:L8"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="E3:F3"/>
-    <mergeCell ref="G3:I3"/>
-    <mergeCell ref="J3:L3"/>
-    <mergeCell ref="M3:Q3"/>
-    <mergeCell ref="R3:R7"/>
-    <mergeCell ref="G4:I4"/>
-    <mergeCell ref="J4:L4"/>
-    <mergeCell ref="M4:Q4"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="D19:L19"/>
+    <mergeCell ref="N19:R19"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="F20:K20"/>
+    <mergeCell ref="N20:R20"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="J17:L17"/>
+    <mergeCell ref="N17:O17"/>
+    <mergeCell ref="P17:R17"/>
+    <mergeCell ref="G18:I18"/>
+    <mergeCell ref="J18:L18"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="F23:K23"/>
+    <mergeCell ref="N23:R23"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="F24:K24"/>
+    <mergeCell ref="N24:R24"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="F21:K21"/>
+    <mergeCell ref="N21:R21"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="F22:K22"/>
+    <mergeCell ref="N22:R22"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="F27:K27"/>
+    <mergeCell ref="N27:R27"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="F28:K28"/>
+    <mergeCell ref="N28:R28"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="F25:K25"/>
+    <mergeCell ref="N25:R25"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="F26:K26"/>
+    <mergeCell ref="N26:R26"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="F31:K31"/>
+    <mergeCell ref="N31:R31"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="F32:K32"/>
+    <mergeCell ref="N32:R32"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="F29:K29"/>
+    <mergeCell ref="N29:R29"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="F30:K30"/>
+    <mergeCell ref="N30:R30"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="F35:K35"/>
+    <mergeCell ref="N35:R35"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="F36:K36"/>
+    <mergeCell ref="N36:R36"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="F33:K33"/>
+    <mergeCell ref="N33:R33"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="F34:K34"/>
+    <mergeCell ref="N34:R34"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="F39:K39"/>
+    <mergeCell ref="N39:R39"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="F40:K40"/>
+    <mergeCell ref="N40:R40"/>
+    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="F37:K37"/>
+    <mergeCell ref="N37:R37"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="F38:K38"/>
+    <mergeCell ref="N38:R38"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="F43:K43"/>
+    <mergeCell ref="N43:R43"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="F44:K44"/>
+    <mergeCell ref="N44:R44"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="F41:K41"/>
+    <mergeCell ref="N41:R41"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="F42:K42"/>
+    <mergeCell ref="N42:R42"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="F47:K47"/>
+    <mergeCell ref="N47:R47"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="F48:K48"/>
+    <mergeCell ref="N48:R48"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="F45:K45"/>
+    <mergeCell ref="N45:R45"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="F46:K46"/>
+    <mergeCell ref="N46:R46"/>
+    <mergeCell ref="D51:E51"/>
+    <mergeCell ref="F51:K51"/>
+    <mergeCell ref="N51:R51"/>
+    <mergeCell ref="D52:E52"/>
+    <mergeCell ref="F52:K52"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="F49:K49"/>
+    <mergeCell ref="N49:R49"/>
+    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="F50:K50"/>
+    <mergeCell ref="N50:R50"/>
+    <mergeCell ref="N52:R52"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Fix : Correcta funcionalidad del excel de HCI
</commit_message>
<xml_diff>
--- a/SupervisorMobility.API/DataAccess/Templates/HCI Template.xlsx
+++ b/SupervisorMobility.API/DataAccess/Templates/HCI Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\job\Supervisor app\Server\SupervisorMobility.API\DataAccess\Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\source\repos\SupervisorMobility.API\SupervisorMobility.API\DataAccess\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C8C37F8-521F-4A35-A1C9-FC777A35B168}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1184C997-8FC6-4B8C-888E-9D773A61D4E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38775" yWindow="3420" windowWidth="24360" windowHeight="15840" xr2:uid="{04842937-1B74-41D6-BD72-7F55AB7A96D5}"/>
+    <workbookView xWindow="32640" yWindow="3840" windowWidth="21600" windowHeight="11835" xr2:uid="{04842937-1B74-41D6-BD72-7F55AB7A96D5}"/>
   </bookViews>
   <sheets>
     <sheet name="HCI" sheetId="1" r:id="rId1"/>
@@ -126,7 +126,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -189,6 +189,13 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -975,45 +982,173 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1021,16 +1156,22 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1040,10 +1181,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1057,160 +1195,49 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1773,105 +1800,105 @@
         <v>0</v>
       </c>
       <c r="B3" s="3"/>
-      <c r="C3" s="89" t="s">
+      <c r="C3" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="90"/>
-      <c r="E3" s="91"/>
-      <c r="F3" s="92"/>
-      <c r="G3" s="93" t="s">
+      <c r="D3" s="39"/>
+      <c r="E3" s="40"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="94"/>
-      <c r="I3" s="94"/>
-      <c r="J3" s="95"/>
-      <c r="K3" s="95"/>
-      <c r="L3" s="96"/>
-      <c r="M3" s="97" t="s">
+      <c r="H3" s="43"/>
+      <c r="I3" s="43"/>
+      <c r="J3" s="44"/>
+      <c r="K3" s="44"/>
+      <c r="L3" s="45"/>
+      <c r="M3" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="N3" s="98"/>
-      <c r="O3" s="98"/>
-      <c r="P3" s="98"/>
-      <c r="Q3" s="98"/>
-      <c r="R3" s="99"/>
+      <c r="N3" s="47"/>
+      <c r="O3" s="47"/>
+      <c r="P3" s="47"/>
+      <c r="Q3" s="47"/>
+      <c r="R3" s="48"/>
     </row>
     <row r="4" spans="1:18" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="42"/>
+      <c r="B4" s="31"/>
       <c r="C4" s="5" t="s">
         <v>5</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="7"/>
-      <c r="F4" s="43"/>
-      <c r="G4" s="102" t="s">
+      <c r="F4" s="32"/>
+      <c r="G4" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="103"/>
-      <c r="I4" s="103"/>
-      <c r="J4" s="104"/>
-      <c r="K4" s="104"/>
-      <c r="L4" s="105"/>
-      <c r="M4" s="106"/>
-      <c r="N4" s="106"/>
-      <c r="O4" s="106"/>
-      <c r="P4" s="106"/>
-      <c r="Q4" s="106"/>
-      <c r="R4" s="100"/>
+      <c r="H4" s="52"/>
+      <c r="I4" s="52"/>
+      <c r="J4" s="53"/>
+      <c r="K4" s="53"/>
+      <c r="L4" s="54"/>
+      <c r="M4" s="55"/>
+      <c r="N4" s="55"/>
+      <c r="O4" s="55"/>
+      <c r="P4" s="55"/>
+      <c r="Q4" s="55"/>
+      <c r="R4" s="49"/>
     </row>
     <row r="5" spans="1:18" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="81" t="s">
+      <c r="A5" s="69" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="81"/>
-      <c r="C5" s="81" t="s">
+      <c r="B5" s="69"/>
+      <c r="C5" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="81"/>
-      <c r="E5" s="81"/>
-      <c r="F5" s="81"/>
-      <c r="G5" s="81"/>
-      <c r="H5" s="81"/>
-      <c r="I5" s="81"/>
-      <c r="J5" s="81"/>
-      <c r="K5" s="81"/>
-      <c r="L5" s="81"/>
-      <c r="R5" s="100"/>
+      <c r="D5" s="69"/>
+      <c r="E5" s="69"/>
+      <c r="F5" s="69"/>
+      <c r="G5" s="69"/>
+      <c r="H5" s="69"/>
+      <c r="I5" s="69"/>
+      <c r="J5" s="69"/>
+      <c r="K5" s="69"/>
+      <c r="L5" s="69"/>
+      <c r="R5" s="49"/>
     </row>
     <row r="6" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="82" t="s">
+      <c r="A6" s="70" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="83"/>
-      <c r="D6" s="82" t="s">
+      <c r="B6" s="71"/>
+      <c r="D6" s="70" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="86"/>
-      <c r="F6" s="86"/>
-      <c r="G6" s="86"/>
-      <c r="H6" s="86"/>
-      <c r="I6" s="86"/>
-      <c r="J6" s="86"/>
-      <c r="K6" s="86"/>
-      <c r="L6" s="83"/>
-      <c r="R6" s="100"/>
+      <c r="E6" s="74"/>
+      <c r="F6" s="74"/>
+      <c r="G6" s="74"/>
+      <c r="H6" s="74"/>
+      <c r="I6" s="74"/>
+      <c r="J6" s="74"/>
+      <c r="K6" s="74"/>
+      <c r="L6" s="71"/>
+      <c r="R6" s="49"/>
     </row>
     <row r="7" spans="1:18" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="84"/>
-      <c r="B7" s="85"/>
-      <c r="D7" s="84"/>
-      <c r="E7" s="87"/>
-      <c r="F7" s="87"/>
-      <c r="G7" s="87"/>
-      <c r="H7" s="87"/>
-      <c r="I7" s="87"/>
-      <c r="J7" s="87"/>
-      <c r="K7" s="87"/>
-      <c r="L7" s="85"/>
-      <c r="R7" s="101"/>
+      <c r="A7" s="72"/>
+      <c r="B7" s="73"/>
+      <c r="D7" s="72"/>
+      <c r="E7" s="75"/>
+      <c r="F7" s="75"/>
+      <c r="G7" s="75"/>
+      <c r="H7" s="75"/>
+      <c r="I7" s="75"/>
+      <c r="J7" s="75"/>
+      <c r="K7" s="75"/>
+      <c r="L7" s="73"/>
+      <c r="R7" s="50"/>
     </row>
     <row r="8" spans="1:18" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="8" t="s">
@@ -1889,33 +1916,33 @@
       <c r="F8" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="G8" s="69" t="s">
+      <c r="G8" s="76" t="s">
         <v>16</v>
       </c>
-      <c r="H8" s="70"/>
-      <c r="I8" s="68"/>
-      <c r="J8" s="69" t="s">
+      <c r="H8" s="77"/>
+      <c r="I8" s="78"/>
+      <c r="J8" s="76" t="s">
         <v>17</v>
       </c>
-      <c r="K8" s="70"/>
-      <c r="L8" s="88"/>
+      <c r="K8" s="77"/>
+      <c r="L8" s="79"/>
     </row>
     <row r="9" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="109"/>
-      <c r="B9" s="24"/>
-      <c r="D9" s="31"/>
-      <c r="E9" s="32"/>
-      <c r="F9" s="32"/>
-      <c r="G9" s="78"/>
-      <c r="H9" s="71"/>
-      <c r="I9" s="59"/>
-      <c r="J9" s="78"/>
-      <c r="K9" s="71"/>
-      <c r="L9" s="72"/>
-      <c r="N9" s="79" t="s">
+      <c r="A9" s="37"/>
+      <c r="B9" s="96"/>
+      <c r="D9" s="108"/>
+      <c r="E9" s="109"/>
+      <c r="F9" s="109"/>
+      <c r="G9" s="56"/>
+      <c r="H9" s="57"/>
+      <c r="I9" s="58"/>
+      <c r="J9" s="56"/>
+      <c r="K9" s="57"/>
+      <c r="L9" s="59"/>
+      <c r="N9" s="60" t="s">
         <v>18</v>
       </c>
-      <c r="O9" s="80"/>
+      <c r="O9" s="61"/>
       <c r="P9" s="13" t="s">
         <v>19</v>
       </c>
@@ -1923,215 +1950,215 @@
       <c r="R9" s="15"/>
     </row>
     <row r="10" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="25"/>
-      <c r="B10" s="26"/>
+      <c r="A10" s="24"/>
+      <c r="B10" s="25"/>
       <c r="C10" s="16"/>
-      <c r="D10" s="33"/>
-      <c r="E10" s="34"/>
-      <c r="F10" s="35"/>
-      <c r="G10" s="73"/>
-      <c r="H10" s="74"/>
-      <c r="I10" s="75"/>
-      <c r="J10" s="76"/>
-      <c r="K10" s="48"/>
-      <c r="L10" s="49"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="33"/>
+      <c r="G10" s="62"/>
+      <c r="H10" s="63"/>
+      <c r="I10" s="64"/>
+      <c r="J10" s="65"/>
+      <c r="K10" s="66"/>
+      <c r="L10" s="67"/>
       <c r="M10" s="17"/>
-      <c r="N10" s="58"/>
-      <c r="O10" s="59"/>
-      <c r="P10" s="78"/>
-      <c r="Q10" s="71"/>
-      <c r="R10" s="72"/>
+      <c r="N10" s="68"/>
+      <c r="O10" s="58"/>
+      <c r="P10" s="56"/>
+      <c r="Q10" s="57"/>
+      <c r="R10" s="59"/>
     </row>
     <row r="11" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="25"/>
-      <c r="B11" s="26"/>
+      <c r="A11" s="24"/>
+      <c r="B11" s="25"/>
       <c r="C11" s="16"/>
-      <c r="D11" s="33"/>
-      <c r="E11" s="34"/>
-      <c r="F11" s="36"/>
-      <c r="G11" s="73"/>
-      <c r="H11" s="74"/>
-      <c r="I11" s="75"/>
-      <c r="J11" s="76"/>
-      <c r="K11" s="48"/>
-      <c r="L11" s="49"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="28"/>
+      <c r="G11" s="62"/>
+      <c r="H11" s="63"/>
+      <c r="I11" s="64"/>
+      <c r="J11" s="65"/>
+      <c r="K11" s="66"/>
+      <c r="L11" s="67"/>
       <c r="M11" s="18"/>
-      <c r="N11" s="44"/>
-      <c r="O11" s="45"/>
-      <c r="P11" s="76" t="s">
+      <c r="N11" s="80"/>
+      <c r="O11" s="81"/>
+      <c r="P11" s="65" t="s">
         <v>20</v>
       </c>
-      <c r="Q11" s="48"/>
-      <c r="R11" s="49"/>
+      <c r="Q11" s="66"/>
+      <c r="R11" s="67"/>
     </row>
     <row r="12" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="107" t="s">
+      <c r="A12" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="28"/>
-      <c r="D12" s="27"/>
-      <c r="E12" s="37"/>
-      <c r="F12" s="37"/>
-      <c r="G12" s="73"/>
-      <c r="H12" s="74"/>
-      <c r="I12" s="75"/>
-      <c r="J12" s="76"/>
-      <c r="K12" s="48"/>
-      <c r="L12" s="49"/>
-      <c r="N12" s="44"/>
-      <c r="O12" s="45"/>
-      <c r="P12" s="76" t="s">
+      <c r="B12" s="97"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="33"/>
+      <c r="F12" s="33"/>
+      <c r="G12" s="62"/>
+      <c r="H12" s="63"/>
+      <c r="I12" s="64"/>
+      <c r="J12" s="65"/>
+      <c r="K12" s="66"/>
+      <c r="L12" s="67"/>
+      <c r="N12" s="80"/>
+      <c r="O12" s="81"/>
+      <c r="P12" s="65" t="s">
         <v>20</v>
       </c>
-      <c r="Q12" s="48"/>
-      <c r="R12" s="49"/>
+      <c r="Q12" s="66"/>
+      <c r="R12" s="67"/>
     </row>
     <row r="13" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="107"/>
-      <c r="B13" s="29"/>
-      <c r="D13" s="27"/>
-      <c r="E13" s="37"/>
-      <c r="F13" s="37"/>
-      <c r="G13" s="73"/>
-      <c r="H13" s="74"/>
-      <c r="I13" s="75"/>
-      <c r="J13" s="76"/>
-      <c r="K13" s="48"/>
-      <c r="L13" s="49"/>
-      <c r="N13" s="44"/>
-      <c r="O13" s="45"/>
-      <c r="P13" s="76" t="s">
+      <c r="A13" s="35"/>
+      <c r="B13" s="98"/>
+      <c r="D13" s="35"/>
+      <c r="E13" s="33"/>
+      <c r="F13" s="33"/>
+      <c r="G13" s="62"/>
+      <c r="H13" s="63"/>
+      <c r="I13" s="64"/>
+      <c r="J13" s="65"/>
+      <c r="K13" s="66"/>
+      <c r="L13" s="67"/>
+      <c r="N13" s="80"/>
+      <c r="O13" s="81"/>
+      <c r="P13" s="65" t="s">
         <v>20</v>
       </c>
-      <c r="Q13" s="48"/>
-      <c r="R13" s="49"/>
+      <c r="Q13" s="66"/>
+      <c r="R13" s="67"/>
     </row>
     <row r="14" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="107" t="s">
+      <c r="A14" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="28"/>
-      <c r="D14" s="27"/>
-      <c r="E14" s="37"/>
-      <c r="F14" s="37"/>
-      <c r="G14" s="73"/>
-      <c r="H14" s="74"/>
-      <c r="I14" s="75"/>
-      <c r="J14" s="76"/>
-      <c r="K14" s="48"/>
-      <c r="L14" s="49"/>
+      <c r="B14" s="97"/>
+      <c r="D14" s="35"/>
+      <c r="E14" s="33"/>
+      <c r="F14" s="33"/>
+      <c r="G14" s="62"/>
+      <c r="H14" s="63"/>
+      <c r="I14" s="64"/>
+      <c r="J14" s="65"/>
+      <c r="K14" s="66"/>
+      <c r="L14" s="67"/>
       <c r="M14" t="s">
         <v>20</v>
       </c>
-      <c r="N14" s="44"/>
-      <c r="O14" s="45"/>
-      <c r="P14" s="76" t="s">
+      <c r="N14" s="80"/>
+      <c r="O14" s="81"/>
+      <c r="P14" s="65" t="s">
         <v>20</v>
       </c>
-      <c r="Q14" s="48"/>
-      <c r="R14" s="49"/>
+      <c r="Q14" s="66"/>
+      <c r="R14" s="67"/>
     </row>
     <row r="15" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="107" t="s">
+      <c r="A15" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="28"/>
-      <c r="D15" s="27"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="37"/>
-      <c r="G15" s="73"/>
-      <c r="H15" s="74"/>
-      <c r="I15" s="75"/>
-      <c r="J15" s="76"/>
-      <c r="K15" s="48"/>
-      <c r="L15" s="49"/>
+      <c r="B15" s="97"/>
+      <c r="D15" s="35"/>
+      <c r="E15" s="33"/>
+      <c r="F15" s="33"/>
+      <c r="G15" s="62"/>
+      <c r="H15" s="63"/>
+      <c r="I15" s="64"/>
+      <c r="J15" s="65"/>
+      <c r="K15" s="66"/>
+      <c r="L15" s="67"/>
       <c r="M15" t="s">
         <v>20</v>
       </c>
-      <c r="N15" s="44"/>
-      <c r="O15" s="45"/>
-      <c r="P15" s="76" t="s">
+      <c r="N15" s="80"/>
+      <c r="O15" s="81"/>
+      <c r="P15" s="65" t="s">
         <v>20</v>
       </c>
-      <c r="Q15" s="48"/>
-      <c r="R15" s="49"/>
+      <c r="Q15" s="66"/>
+      <c r="R15" s="67"/>
     </row>
     <row r="16" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="107"/>
-      <c r="B16" s="28"/>
-      <c r="D16" s="27"/>
-      <c r="E16" s="37"/>
-      <c r="F16" s="37"/>
-      <c r="G16" s="73"/>
-      <c r="H16" s="74"/>
-      <c r="I16" s="75"/>
-      <c r="J16" s="76"/>
-      <c r="K16" s="48"/>
-      <c r="L16" s="49"/>
-      <c r="N16" s="44"/>
-      <c r="O16" s="45"/>
-      <c r="P16" s="76" t="s">
+      <c r="A16" s="35"/>
+      <c r="B16" s="97"/>
+      <c r="D16" s="35"/>
+      <c r="E16" s="33"/>
+      <c r="F16" s="33"/>
+      <c r="G16" s="62"/>
+      <c r="H16" s="63"/>
+      <c r="I16" s="64"/>
+      <c r="J16" s="65"/>
+      <c r="K16" s="66"/>
+      <c r="L16" s="67"/>
+      <c r="N16" s="80"/>
+      <c r="O16" s="81"/>
+      <c r="P16" s="65" t="s">
         <v>20</v>
       </c>
-      <c r="Q16" s="48"/>
-      <c r="R16" s="49"/>
+      <c r="Q16" s="66"/>
+      <c r="R16" s="67"/>
     </row>
     <row r="17" spans="1:18" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="107"/>
-      <c r="B17" s="28"/>
-      <c r="D17" s="27"/>
-      <c r="E17" s="37"/>
-      <c r="F17" s="37"/>
-      <c r="G17" s="73"/>
-      <c r="H17" s="74"/>
-      <c r="I17" s="75"/>
-      <c r="J17" s="76"/>
-      <c r="K17" s="48"/>
-      <c r="L17" s="49"/>
-      <c r="N17" s="50"/>
-      <c r="O17" s="51"/>
-      <c r="P17" s="77" t="s">
+      <c r="A17" s="35"/>
+      <c r="B17" s="97"/>
+      <c r="D17" s="35"/>
+      <c r="E17" s="33"/>
+      <c r="F17" s="33"/>
+      <c r="G17" s="62"/>
+      <c r="H17" s="63"/>
+      <c r="I17" s="64"/>
+      <c r="J17" s="65"/>
+      <c r="K17" s="66"/>
+      <c r="L17" s="67"/>
+      <c r="N17" s="88"/>
+      <c r="O17" s="89"/>
+      <c r="P17" s="90" t="s">
         <v>20</v>
       </c>
-      <c r="Q17" s="54"/>
-      <c r="R17" s="55"/>
+      <c r="Q17" s="91"/>
+      <c r="R17" s="92"/>
     </row>
     <row r="18" spans="1:18" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="108"/>
-      <c r="B18" s="30"/>
-      <c r="D18" s="27"/>
-      <c r="E18" s="37"/>
-      <c r="F18" s="37"/>
-      <c r="G18" s="73"/>
-      <c r="H18" s="74"/>
-      <c r="I18" s="75"/>
-      <c r="J18" s="76"/>
-      <c r="K18" s="48"/>
-      <c r="L18" s="49"/>
+      <c r="A18" s="36"/>
+      <c r="B18" s="99"/>
+      <c r="D18" s="35"/>
+      <c r="E18" s="33"/>
+      <c r="F18" s="33"/>
+      <c r="G18" s="62"/>
+      <c r="H18" s="63"/>
+      <c r="I18" s="64"/>
+      <c r="J18" s="65"/>
+      <c r="K18" s="66"/>
+      <c r="L18" s="67"/>
     </row>
     <row r="19" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="62" t="s">
+      <c r="A19" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="B19" s="63"/>
-      <c r="D19" s="64" t="s">
+      <c r="B19" s="83"/>
+      <c r="D19" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="E19" s="65"/>
-      <c r="F19" s="65"/>
-      <c r="G19" s="65"/>
-      <c r="H19" s="65"/>
-      <c r="I19" s="65"/>
-      <c r="J19" s="65"/>
-      <c r="K19" s="65"/>
-      <c r="L19" s="66"/>
-      <c r="N19" s="64" t="s">
+      <c r="E19" s="85"/>
+      <c r="F19" s="85"/>
+      <c r="G19" s="85"/>
+      <c r="H19" s="85"/>
+      <c r="I19" s="85"/>
+      <c r="J19" s="85"/>
+      <c r="K19" s="85"/>
+      <c r="L19" s="86"/>
+      <c r="N19" s="84" t="s">
         <v>23</v>
       </c>
-      <c r="O19" s="65"/>
-      <c r="P19" s="65"/>
-      <c r="Q19" s="65"/>
-      <c r="R19" s="66"/>
+      <c r="O19" s="85"/>
+      <c r="P19" s="85"/>
+      <c r="Q19" s="85"/>
+      <c r="R19" s="86"/>
     </row>
     <row r="20" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="19" t="s">
@@ -2140,370 +2167,370 @@
       <c r="B20" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D20" s="67" t="s">
+      <c r="D20" s="87" t="s">
         <v>24</v>
       </c>
-      <c r="E20" s="68"/>
-      <c r="F20" s="69" t="s">
+      <c r="E20" s="78"/>
+      <c r="F20" s="76" t="s">
         <v>17</v>
       </c>
-      <c r="G20" s="70"/>
-      <c r="H20" s="70"/>
-      <c r="I20" s="70"/>
-      <c r="J20" s="70"/>
-      <c r="K20" s="70"/>
+      <c r="G20" s="77"/>
+      <c r="H20" s="77"/>
+      <c r="I20" s="77"/>
+      <c r="J20" s="77"/>
+      <c r="K20" s="77"/>
       <c r="L20" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="N20" s="58"/>
-      <c r="O20" s="71"/>
-      <c r="P20" s="71"/>
-      <c r="Q20" s="71"/>
-      <c r="R20" s="72"/>
+      <c r="N20" s="68"/>
+      <c r="O20" s="57"/>
+      <c r="P20" s="57"/>
+      <c r="Q20" s="57"/>
+      <c r="R20" s="59"/>
     </row>
     <row r="21" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="107"/>
-      <c r="B21" s="28"/>
-      <c r="D21" s="58"/>
-      <c r="E21" s="59"/>
-      <c r="F21" s="60"/>
-      <c r="G21" s="61"/>
-      <c r="H21" s="61"/>
-      <c r="I21" s="61"/>
-      <c r="J21" s="61"/>
-      <c r="K21" s="61"/>
-      <c r="L21" s="38"/>
-      <c r="N21" s="44"/>
-      <c r="O21" s="48"/>
-      <c r="P21" s="48"/>
-      <c r="Q21" s="48"/>
-      <c r="R21" s="49"/>
+      <c r="A21" s="35"/>
+      <c r="B21" s="97"/>
+      <c r="D21" s="68"/>
+      <c r="E21" s="58"/>
+      <c r="F21" s="100"/>
+      <c r="G21" s="101"/>
+      <c r="H21" s="101"/>
+      <c r="I21" s="101"/>
+      <c r="J21" s="101"/>
+      <c r="K21" s="101"/>
+      <c r="L21" s="29"/>
+      <c r="N21" s="80"/>
+      <c r="O21" s="66"/>
+      <c r="P21" s="66"/>
+      <c r="Q21" s="66"/>
+      <c r="R21" s="67"/>
     </row>
     <row r="22" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="107"/>
-      <c r="B22" s="28"/>
-      <c r="D22" s="44"/>
-      <c r="E22" s="45"/>
-      <c r="F22" s="46"/>
-      <c r="G22" s="47"/>
-      <c r="H22" s="47"/>
-      <c r="I22" s="47"/>
-      <c r="J22" s="47"/>
-      <c r="K22" s="47"/>
-      <c r="L22" s="39"/>
-      <c r="N22" s="44"/>
-      <c r="O22" s="48"/>
-      <c r="P22" s="48"/>
-      <c r="Q22" s="48"/>
-      <c r="R22" s="49"/>
+      <c r="A22" s="35"/>
+      <c r="B22" s="97"/>
+      <c r="D22" s="80"/>
+      <c r="E22" s="81"/>
+      <c r="F22" s="102"/>
+      <c r="G22" s="103"/>
+      <c r="H22" s="103"/>
+      <c r="I22" s="103"/>
+      <c r="J22" s="103"/>
+      <c r="K22" s="103"/>
+      <c r="L22" s="30"/>
+      <c r="N22" s="80"/>
+      <c r="O22" s="66"/>
+      <c r="P22" s="66"/>
+      <c r="Q22" s="66"/>
+      <c r="R22" s="67"/>
     </row>
     <row r="23" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="107"/>
-      <c r="B23" s="28"/>
-      <c r="D23" s="44"/>
-      <c r="E23" s="45"/>
-      <c r="F23" s="46"/>
-      <c r="G23" s="47"/>
-      <c r="H23" s="47"/>
-      <c r="I23" s="47"/>
-      <c r="J23" s="47"/>
-      <c r="K23" s="47"/>
-      <c r="L23" s="39"/>
-      <c r="N23" s="44"/>
-      <c r="O23" s="48"/>
-      <c r="P23" s="48"/>
-      <c r="Q23" s="48"/>
-      <c r="R23" s="49"/>
+      <c r="A23" s="35"/>
+      <c r="B23" s="97"/>
+      <c r="D23" s="80"/>
+      <c r="E23" s="81"/>
+      <c r="F23" s="102"/>
+      <c r="G23" s="103"/>
+      <c r="H23" s="103"/>
+      <c r="I23" s="103"/>
+      <c r="J23" s="103"/>
+      <c r="K23" s="103"/>
+      <c r="L23" s="30"/>
+      <c r="N23" s="80"/>
+      <c r="O23" s="66"/>
+      <c r="P23" s="66"/>
+      <c r="Q23" s="66"/>
+      <c r="R23" s="67"/>
     </row>
     <row r="24" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="107"/>
-      <c r="B24" s="28"/>
-      <c r="D24" s="44"/>
-      <c r="E24" s="45"/>
-      <c r="F24" s="46"/>
-      <c r="G24" s="47"/>
-      <c r="H24" s="47"/>
-      <c r="I24" s="47"/>
-      <c r="J24" s="47"/>
-      <c r="K24" s="47"/>
-      <c r="L24" s="39"/>
-      <c r="N24" s="44"/>
-      <c r="O24" s="48"/>
-      <c r="P24" s="48"/>
-      <c r="Q24" s="48"/>
-      <c r="R24" s="49"/>
+      <c r="A24" s="35"/>
+      <c r="B24" s="97"/>
+      <c r="D24" s="80"/>
+      <c r="E24" s="81"/>
+      <c r="F24" s="102"/>
+      <c r="G24" s="103"/>
+      <c r="H24" s="103"/>
+      <c r="I24" s="103"/>
+      <c r="J24" s="103"/>
+      <c r="K24" s="103"/>
+      <c r="L24" s="30"/>
+      <c r="N24" s="80"/>
+      <c r="O24" s="66"/>
+      <c r="P24" s="66"/>
+      <c r="Q24" s="66"/>
+      <c r="R24" s="67"/>
     </row>
     <row r="25" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="107"/>
-      <c r="B25" s="28"/>
-      <c r="D25" s="44"/>
-      <c r="E25" s="45"/>
-      <c r="F25" s="46"/>
-      <c r="G25" s="47"/>
-      <c r="H25" s="47"/>
-      <c r="I25" s="47"/>
-      <c r="J25" s="47"/>
-      <c r="K25" s="47"/>
-      <c r="L25" s="39"/>
-      <c r="N25" s="44"/>
-      <c r="O25" s="48"/>
-      <c r="P25" s="48"/>
-      <c r="Q25" s="48"/>
-      <c r="R25" s="49"/>
+      <c r="A25" s="35"/>
+      <c r="B25" s="97"/>
+      <c r="D25" s="80"/>
+      <c r="E25" s="81"/>
+      <c r="F25" s="102"/>
+      <c r="G25" s="103"/>
+      <c r="H25" s="103"/>
+      <c r="I25" s="103"/>
+      <c r="J25" s="103"/>
+      <c r="K25" s="103"/>
+      <c r="L25" s="30"/>
+      <c r="N25" s="80"/>
+      <c r="O25" s="66"/>
+      <c r="P25" s="66"/>
+      <c r="Q25" s="66"/>
+      <c r="R25" s="67"/>
     </row>
     <row r="26" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="107"/>
-      <c r="B26" s="28"/>
-      <c r="D26" s="44"/>
-      <c r="E26" s="45"/>
-      <c r="F26" s="46"/>
-      <c r="G26" s="47"/>
-      <c r="H26" s="47"/>
-      <c r="I26" s="47"/>
-      <c r="J26" s="47"/>
-      <c r="K26" s="47"/>
-      <c r="L26" s="39"/>
-      <c r="N26" s="44"/>
-      <c r="O26" s="48"/>
-      <c r="P26" s="48"/>
-      <c r="Q26" s="48"/>
-      <c r="R26" s="49"/>
+      <c r="A26" s="35"/>
+      <c r="B26" s="97"/>
+      <c r="D26" s="80"/>
+      <c r="E26" s="81"/>
+      <c r="F26" s="102"/>
+      <c r="G26" s="103"/>
+      <c r="H26" s="103"/>
+      <c r="I26" s="103"/>
+      <c r="J26" s="103"/>
+      <c r="K26" s="103"/>
+      <c r="L26" s="30"/>
+      <c r="N26" s="80"/>
+      <c r="O26" s="66"/>
+      <c r="P26" s="66"/>
+      <c r="Q26" s="66"/>
+      <c r="R26" s="67"/>
     </row>
     <row r="27" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="107"/>
-      <c r="B27" s="28"/>
-      <c r="D27" s="44"/>
-      <c r="E27" s="45"/>
-      <c r="F27" s="46"/>
-      <c r="G27" s="47"/>
-      <c r="H27" s="47"/>
-      <c r="I27" s="47"/>
-      <c r="J27" s="47"/>
-      <c r="K27" s="47"/>
-      <c r="L27" s="39"/>
-      <c r="N27" s="44"/>
-      <c r="O27" s="48"/>
-      <c r="P27" s="48"/>
-      <c r="Q27" s="48"/>
-      <c r="R27" s="49"/>
+      <c r="A27" s="35"/>
+      <c r="B27" s="97"/>
+      <c r="D27" s="80"/>
+      <c r="E27" s="81"/>
+      <c r="F27" s="102"/>
+      <c r="G27" s="103"/>
+      <c r="H27" s="103"/>
+      <c r="I27" s="103"/>
+      <c r="J27" s="103"/>
+      <c r="K27" s="103"/>
+      <c r="L27" s="30"/>
+      <c r="N27" s="80"/>
+      <c r="O27" s="66"/>
+      <c r="P27" s="66"/>
+      <c r="Q27" s="66"/>
+      <c r="R27" s="67"/>
     </row>
     <row r="28" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="107"/>
-      <c r="B28" s="28"/>
-      <c r="D28" s="44"/>
-      <c r="E28" s="45"/>
-      <c r="F28" s="46"/>
-      <c r="G28" s="47"/>
-      <c r="H28" s="47"/>
-      <c r="I28" s="47"/>
-      <c r="J28" s="47"/>
-      <c r="K28" s="47"/>
-      <c r="L28" s="39"/>
-      <c r="N28" s="44"/>
-      <c r="O28" s="48"/>
-      <c r="P28" s="48"/>
-      <c r="Q28" s="48"/>
-      <c r="R28" s="49"/>
+      <c r="A28" s="35"/>
+      <c r="B28" s="97"/>
+      <c r="D28" s="80"/>
+      <c r="E28" s="81"/>
+      <c r="F28" s="102"/>
+      <c r="G28" s="103"/>
+      <c r="H28" s="103"/>
+      <c r="I28" s="103"/>
+      <c r="J28" s="103"/>
+      <c r="K28" s="103"/>
+      <c r="L28" s="30"/>
+      <c r="N28" s="80"/>
+      <c r="O28" s="66"/>
+      <c r="P28" s="66"/>
+      <c r="Q28" s="66"/>
+      <c r="R28" s="67"/>
     </row>
     <row r="29" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="107"/>
-      <c r="B29" s="28"/>
-      <c r="D29" s="44"/>
-      <c r="E29" s="45"/>
-      <c r="F29" s="46"/>
-      <c r="G29" s="47"/>
-      <c r="H29" s="47"/>
-      <c r="I29" s="47"/>
-      <c r="J29" s="47"/>
-      <c r="K29" s="47"/>
-      <c r="L29" s="39"/>
-      <c r="N29" s="44"/>
-      <c r="O29" s="48"/>
-      <c r="P29" s="48"/>
-      <c r="Q29" s="48"/>
-      <c r="R29" s="49"/>
+      <c r="A29" s="35"/>
+      <c r="B29" s="97"/>
+      <c r="D29" s="80"/>
+      <c r="E29" s="81"/>
+      <c r="F29" s="102"/>
+      <c r="G29" s="103"/>
+      <c r="H29" s="103"/>
+      <c r="I29" s="103"/>
+      <c r="J29" s="103"/>
+      <c r="K29" s="103"/>
+      <c r="L29" s="30"/>
+      <c r="N29" s="80"/>
+      <c r="O29" s="66"/>
+      <c r="P29" s="66"/>
+      <c r="Q29" s="66"/>
+      <c r="R29" s="67"/>
     </row>
     <row r="30" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="107"/>
-      <c r="B30" s="28"/>
-      <c r="D30" s="44"/>
-      <c r="E30" s="45"/>
-      <c r="F30" s="46"/>
-      <c r="G30" s="47"/>
-      <c r="H30" s="47"/>
-      <c r="I30" s="47"/>
-      <c r="J30" s="47"/>
-      <c r="K30" s="47"/>
-      <c r="L30" s="39"/>
-      <c r="N30" s="44"/>
-      <c r="O30" s="48"/>
-      <c r="P30" s="48"/>
-      <c r="Q30" s="48"/>
-      <c r="R30" s="49"/>
+      <c r="A30" s="35"/>
+      <c r="B30" s="97"/>
+      <c r="D30" s="80"/>
+      <c r="E30" s="81"/>
+      <c r="F30" s="102"/>
+      <c r="G30" s="103"/>
+      <c r="H30" s="103"/>
+      <c r="I30" s="103"/>
+      <c r="J30" s="103"/>
+      <c r="K30" s="103"/>
+      <c r="L30" s="30"/>
+      <c r="N30" s="80"/>
+      <c r="O30" s="66"/>
+      <c r="P30" s="66"/>
+      <c r="Q30" s="66"/>
+      <c r="R30" s="67"/>
     </row>
     <row r="31" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="107"/>
-      <c r="B31" s="28"/>
-      <c r="D31" s="44"/>
-      <c r="E31" s="45"/>
-      <c r="F31" s="46"/>
-      <c r="G31" s="47"/>
-      <c r="H31" s="47"/>
-      <c r="I31" s="47"/>
-      <c r="J31" s="47"/>
-      <c r="K31" s="47"/>
-      <c r="L31" s="39"/>
-      <c r="N31" s="44"/>
-      <c r="O31" s="48"/>
-      <c r="P31" s="48"/>
-      <c r="Q31" s="48"/>
-      <c r="R31" s="49"/>
+      <c r="A31" s="35"/>
+      <c r="B31" s="97"/>
+      <c r="D31" s="80"/>
+      <c r="E31" s="81"/>
+      <c r="F31" s="102"/>
+      <c r="G31" s="103"/>
+      <c r="H31" s="103"/>
+      <c r="I31" s="103"/>
+      <c r="J31" s="103"/>
+      <c r="K31" s="103"/>
+      <c r="L31" s="30"/>
+      <c r="N31" s="80"/>
+      <c r="O31" s="66"/>
+      <c r="P31" s="66"/>
+      <c r="Q31" s="66"/>
+      <c r="R31" s="67"/>
     </row>
     <row r="32" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="107"/>
-      <c r="B32" s="28"/>
-      <c r="D32" s="44"/>
-      <c r="E32" s="45"/>
-      <c r="F32" s="46"/>
-      <c r="G32" s="47"/>
-      <c r="H32" s="47"/>
-      <c r="I32" s="47"/>
-      <c r="J32" s="47"/>
-      <c r="K32" s="47"/>
-      <c r="L32" s="39"/>
-      <c r="N32" s="44"/>
-      <c r="O32" s="48"/>
-      <c r="P32" s="48"/>
-      <c r="Q32" s="48"/>
-      <c r="R32" s="49"/>
+      <c r="A32" s="35"/>
+      <c r="B32" s="97"/>
+      <c r="D32" s="80"/>
+      <c r="E32" s="81"/>
+      <c r="F32" s="102"/>
+      <c r="G32" s="103"/>
+      <c r="H32" s="103"/>
+      <c r="I32" s="103"/>
+      <c r="J32" s="103"/>
+      <c r="K32" s="103"/>
+      <c r="L32" s="30"/>
+      <c r="N32" s="80"/>
+      <c r="O32" s="66"/>
+      <c r="P32" s="66"/>
+      <c r="Q32" s="66"/>
+      <c r="R32" s="67"/>
     </row>
     <row r="33" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="107"/>
-      <c r="B33" s="28"/>
-      <c r="D33" s="44"/>
-      <c r="E33" s="45"/>
-      <c r="F33" s="46"/>
-      <c r="G33" s="47"/>
-      <c r="H33" s="47"/>
-      <c r="I33" s="47"/>
-      <c r="J33" s="47"/>
-      <c r="K33" s="47"/>
-      <c r="L33" s="39"/>
-      <c r="N33" s="44"/>
-      <c r="O33" s="48"/>
-      <c r="P33" s="48"/>
-      <c r="Q33" s="48"/>
-      <c r="R33" s="49"/>
+      <c r="A33" s="35"/>
+      <c r="B33" s="97"/>
+      <c r="D33" s="80"/>
+      <c r="E33" s="81"/>
+      <c r="F33" s="102"/>
+      <c r="G33" s="103"/>
+      <c r="H33" s="103"/>
+      <c r="I33" s="103"/>
+      <c r="J33" s="103"/>
+      <c r="K33" s="103"/>
+      <c r="L33" s="30"/>
+      <c r="N33" s="80"/>
+      <c r="O33" s="66"/>
+      <c r="P33" s="66"/>
+      <c r="Q33" s="66"/>
+      <c r="R33" s="67"/>
     </row>
     <row r="34" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="107"/>
-      <c r="B34" s="28"/>
-      <c r="D34" s="44"/>
-      <c r="E34" s="45"/>
-      <c r="F34" s="46"/>
-      <c r="G34" s="47"/>
-      <c r="H34" s="47"/>
-      <c r="I34" s="47"/>
-      <c r="J34" s="47"/>
-      <c r="K34" s="47"/>
-      <c r="L34" s="39"/>
-      <c r="N34" s="44"/>
-      <c r="O34" s="48"/>
-      <c r="P34" s="48"/>
-      <c r="Q34" s="48"/>
-      <c r="R34" s="49"/>
+      <c r="A34" s="35"/>
+      <c r="B34" s="97"/>
+      <c r="D34" s="80"/>
+      <c r="E34" s="81"/>
+      <c r="F34" s="102"/>
+      <c r="G34" s="103"/>
+      <c r="H34" s="103"/>
+      <c r="I34" s="103"/>
+      <c r="J34" s="103"/>
+      <c r="K34" s="103"/>
+      <c r="L34" s="30"/>
+      <c r="N34" s="80"/>
+      <c r="O34" s="66"/>
+      <c r="P34" s="66"/>
+      <c r="Q34" s="66"/>
+      <c r="R34" s="67"/>
     </row>
     <row r="35" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="107"/>
-      <c r="B35" s="28"/>
-      <c r="D35" s="44"/>
-      <c r="E35" s="45"/>
-      <c r="F35" s="46"/>
-      <c r="G35" s="47"/>
-      <c r="H35" s="47"/>
-      <c r="I35" s="47"/>
-      <c r="J35" s="47"/>
-      <c r="K35" s="47"/>
-      <c r="L35" s="39"/>
-      <c r="N35" s="44"/>
-      <c r="O35" s="48"/>
-      <c r="P35" s="48"/>
-      <c r="Q35" s="48"/>
-      <c r="R35" s="49"/>
+      <c r="A35" s="35"/>
+      <c r="B35" s="97"/>
+      <c r="D35" s="80"/>
+      <c r="E35" s="81"/>
+      <c r="F35" s="102"/>
+      <c r="G35" s="103"/>
+      <c r="H35" s="103"/>
+      <c r="I35" s="103"/>
+      <c r="J35" s="103"/>
+      <c r="K35" s="103"/>
+      <c r="L35" s="30"/>
+      <c r="N35" s="80"/>
+      <c r="O35" s="66"/>
+      <c r="P35" s="66"/>
+      <c r="Q35" s="66"/>
+      <c r="R35" s="67"/>
     </row>
     <row r="36" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="107"/>
-      <c r="B36" s="28"/>
-      <c r="D36" s="44"/>
-      <c r="E36" s="45"/>
-      <c r="F36" s="46"/>
-      <c r="G36" s="47"/>
-      <c r="H36" s="47"/>
-      <c r="I36" s="47"/>
-      <c r="J36" s="47"/>
-      <c r="K36" s="47"/>
-      <c r="L36" s="39"/>
-      <c r="N36" s="44"/>
-      <c r="O36" s="48"/>
-      <c r="P36" s="48"/>
-      <c r="Q36" s="48"/>
-      <c r="R36" s="49"/>
+      <c r="A36" s="35"/>
+      <c r="B36" s="97"/>
+      <c r="D36" s="80"/>
+      <c r="E36" s="81"/>
+      <c r="F36" s="102"/>
+      <c r="G36" s="103"/>
+      <c r="H36" s="103"/>
+      <c r="I36" s="103"/>
+      <c r="J36" s="103"/>
+      <c r="K36" s="103"/>
+      <c r="L36" s="30"/>
+      <c r="N36" s="80"/>
+      <c r="O36" s="66"/>
+      <c r="P36" s="66"/>
+      <c r="Q36" s="66"/>
+      <c r="R36" s="67"/>
     </row>
     <row r="37" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="107"/>
-      <c r="B37" s="28"/>
-      <c r="D37" s="44"/>
-      <c r="E37" s="45"/>
-      <c r="F37" s="46"/>
-      <c r="G37" s="47"/>
-      <c r="H37" s="47"/>
-      <c r="I37" s="47"/>
-      <c r="J37" s="47"/>
-      <c r="K37" s="47"/>
-      <c r="L37" s="39"/>
-      <c r="N37" s="44"/>
-      <c r="O37" s="48"/>
-      <c r="P37" s="48"/>
-      <c r="Q37" s="48"/>
-      <c r="R37" s="49"/>
+      <c r="A37" s="35"/>
+      <c r="B37" s="97"/>
+      <c r="D37" s="80"/>
+      <c r="E37" s="81"/>
+      <c r="F37" s="102"/>
+      <c r="G37" s="103"/>
+      <c r="H37" s="103"/>
+      <c r="I37" s="103"/>
+      <c r="J37" s="103"/>
+      <c r="K37" s="103"/>
+      <c r="L37" s="30"/>
+      <c r="N37" s="80"/>
+      <c r="O37" s="66"/>
+      <c r="P37" s="66"/>
+      <c r="Q37" s="66"/>
+      <c r="R37" s="67"/>
     </row>
     <row r="38" spans="1:18" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="108"/>
-      <c r="B38" s="30"/>
-      <c r="D38" s="44"/>
-      <c r="E38" s="45"/>
-      <c r="F38" s="46"/>
-      <c r="G38" s="47"/>
-      <c r="H38" s="47"/>
-      <c r="I38" s="47"/>
-      <c r="J38" s="47"/>
-      <c r="K38" s="47"/>
-      <c r="L38" s="39"/>
-      <c r="N38" s="44"/>
-      <c r="O38" s="48"/>
-      <c r="P38" s="48"/>
-      <c r="Q38" s="48"/>
-      <c r="R38" s="49"/>
+      <c r="A38" s="36"/>
+      <c r="B38" s="99"/>
+      <c r="D38" s="80"/>
+      <c r="E38" s="81"/>
+      <c r="F38" s="102"/>
+      <c r="G38" s="103"/>
+      <c r="H38" s="103"/>
+      <c r="I38" s="103"/>
+      <c r="J38" s="103"/>
+      <c r="K38" s="103"/>
+      <c r="L38" s="30"/>
+      <c r="N38" s="80"/>
+      <c r="O38" s="66"/>
+      <c r="P38" s="66"/>
+      <c r="Q38" s="66"/>
+      <c r="R38" s="67"/>
     </row>
     <row r="39" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="56" t="s">
+      <c r="A39" s="93" t="s">
         <v>26</v>
       </c>
-      <c r="B39" s="57"/>
-      <c r="D39" s="44"/>
-      <c r="E39" s="45"/>
-      <c r="F39" s="46"/>
-      <c r="G39" s="47"/>
-      <c r="H39" s="47"/>
-      <c r="I39" s="47"/>
-      <c r="J39" s="47"/>
-      <c r="K39" s="47"/>
-      <c r="L39" s="39"/>
-      <c r="N39" s="44"/>
-      <c r="O39" s="48"/>
-      <c r="P39" s="48"/>
-      <c r="Q39" s="48"/>
-      <c r="R39" s="49"/>
+      <c r="B39" s="94"/>
+      <c r="D39" s="80"/>
+      <c r="E39" s="81"/>
+      <c r="F39" s="102"/>
+      <c r="G39" s="103"/>
+      <c r="H39" s="103"/>
+      <c r="I39" s="103"/>
+      <c r="J39" s="103"/>
+      <c r="K39" s="103"/>
+      <c r="L39" s="30"/>
+      <c r="N39" s="80"/>
+      <c r="O39" s="66"/>
+      <c r="P39" s="66"/>
+      <c r="Q39" s="66"/>
+      <c r="R39" s="67"/>
     </row>
     <row r="40" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="22" t="s">
@@ -2512,270 +2539,349 @@
       <c r="B40" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="D40" s="44"/>
-      <c r="E40" s="45"/>
-      <c r="F40" s="46"/>
-      <c r="G40" s="47"/>
-      <c r="H40" s="47"/>
-      <c r="I40" s="47"/>
-      <c r="J40" s="47"/>
-      <c r="K40" s="47"/>
-      <c r="L40" s="39"/>
-      <c r="N40" s="44"/>
-      <c r="O40" s="48"/>
-      <c r="P40" s="48"/>
-      <c r="Q40" s="48"/>
-      <c r="R40" s="49"/>
+      <c r="D40" s="80"/>
+      <c r="E40" s="81"/>
+      <c r="F40" s="102"/>
+      <c r="G40" s="103"/>
+      <c r="H40" s="103"/>
+      <c r="I40" s="103"/>
+      <c r="J40" s="103"/>
+      <c r="K40" s="103"/>
+      <c r="L40" s="30"/>
+      <c r="N40" s="80"/>
+      <c r="O40" s="66"/>
+      <c r="P40" s="66"/>
+      <c r="Q40" s="66"/>
+      <c r="R40" s="67"/>
     </row>
     <row r="41" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="107"/>
-      <c r="B41" s="28"/>
-      <c r="D41" s="44"/>
-      <c r="E41" s="45"/>
-      <c r="F41" s="46"/>
-      <c r="G41" s="47"/>
-      <c r="H41" s="47"/>
-      <c r="I41" s="47"/>
-      <c r="J41" s="47"/>
-      <c r="K41" s="47"/>
-      <c r="L41" s="39"/>
-      <c r="N41" s="44"/>
-      <c r="O41" s="48"/>
-      <c r="P41" s="48"/>
-      <c r="Q41" s="48"/>
-      <c r="R41" s="49"/>
+      <c r="A41" s="35"/>
+      <c r="B41" s="34"/>
+      <c r="D41" s="80"/>
+      <c r="E41" s="81"/>
+      <c r="F41" s="102"/>
+      <c r="G41" s="103"/>
+      <c r="H41" s="103"/>
+      <c r="I41" s="103"/>
+      <c r="J41" s="103"/>
+      <c r="K41" s="103"/>
+      <c r="L41" s="30"/>
+      <c r="N41" s="80"/>
+      <c r="O41" s="66"/>
+      <c r="P41" s="66"/>
+      <c r="Q41" s="66"/>
+      <c r="R41" s="67"/>
     </row>
     <row r="42" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="107"/>
-      <c r="B42" s="28"/>
-      <c r="D42" s="44"/>
-      <c r="E42" s="45"/>
-      <c r="F42" s="46"/>
-      <c r="G42" s="47"/>
-      <c r="H42" s="47"/>
-      <c r="I42" s="47"/>
-      <c r="J42" s="47"/>
-      <c r="K42" s="47"/>
-      <c r="L42" s="39"/>
-      <c r="N42" s="44"/>
-      <c r="O42" s="48"/>
-      <c r="P42" s="48"/>
-      <c r="Q42" s="48"/>
-      <c r="R42" s="49"/>
+      <c r="A42" s="35"/>
+      <c r="B42" s="34"/>
+      <c r="D42" s="80"/>
+      <c r="E42" s="81"/>
+      <c r="F42" s="102"/>
+      <c r="G42" s="103"/>
+      <c r="H42" s="103"/>
+      <c r="I42" s="103"/>
+      <c r="J42" s="103"/>
+      <c r="K42" s="103"/>
+      <c r="L42" s="30"/>
+      <c r="N42" s="80"/>
+      <c r="O42" s="66"/>
+      <c r="P42" s="66"/>
+      <c r="Q42" s="66"/>
+      <c r="R42" s="67"/>
     </row>
     <row r="43" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="107"/>
-      <c r="B43" s="28"/>
-      <c r="D43" s="44"/>
-      <c r="E43" s="45"/>
-      <c r="F43" s="46"/>
-      <c r="G43" s="47"/>
-      <c r="H43" s="47"/>
-      <c r="I43" s="47"/>
-      <c r="J43" s="47"/>
-      <c r="K43" s="47"/>
-      <c r="L43" s="39"/>
-      <c r="N43" s="44"/>
-      <c r="O43" s="48"/>
-      <c r="P43" s="48"/>
-      <c r="Q43" s="48"/>
-      <c r="R43" s="49"/>
+      <c r="A43" s="35"/>
+      <c r="B43" s="34"/>
+      <c r="D43" s="80"/>
+      <c r="E43" s="81"/>
+      <c r="F43" s="102"/>
+      <c r="G43" s="103"/>
+      <c r="H43" s="103"/>
+      <c r="I43" s="103"/>
+      <c r="J43" s="103"/>
+      <c r="K43" s="103"/>
+      <c r="L43" s="30"/>
+      <c r="N43" s="80"/>
+      <c r="O43" s="66"/>
+      <c r="P43" s="66"/>
+      <c r="Q43" s="66"/>
+      <c r="R43" s="67"/>
     </row>
     <row r="44" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="107"/>
-      <c r="B44" s="28"/>
-      <c r="D44" s="44"/>
-      <c r="E44" s="45"/>
-      <c r="F44" s="46"/>
-      <c r="G44" s="47"/>
-      <c r="H44" s="47"/>
-      <c r="I44" s="47"/>
-      <c r="J44" s="47"/>
-      <c r="K44" s="47"/>
-      <c r="L44" s="39"/>
-      <c r="N44" s="44"/>
-      <c r="O44" s="48"/>
-      <c r="P44" s="48"/>
-      <c r="Q44" s="48"/>
-      <c r="R44" s="49"/>
+      <c r="A44" s="35"/>
+      <c r="B44" s="34"/>
+      <c r="D44" s="80"/>
+      <c r="E44" s="81"/>
+      <c r="F44" s="102"/>
+      <c r="G44" s="103"/>
+      <c r="H44" s="103"/>
+      <c r="I44" s="103"/>
+      <c r="J44" s="103"/>
+      <c r="K44" s="103"/>
+      <c r="L44" s="30"/>
+      <c r="N44" s="80"/>
+      <c r="O44" s="66"/>
+      <c r="P44" s="66"/>
+      <c r="Q44" s="66"/>
+      <c r="R44" s="67"/>
     </row>
     <row r="45" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="107"/>
-      <c r="B45" s="28"/>
-      <c r="D45" s="44"/>
-      <c r="E45" s="45"/>
-      <c r="F45" s="46"/>
-      <c r="G45" s="47"/>
-      <c r="H45" s="47"/>
-      <c r="I45" s="47"/>
-      <c r="J45" s="47"/>
-      <c r="K45" s="47"/>
-      <c r="L45" s="39"/>
-      <c r="N45" s="44"/>
-      <c r="O45" s="48"/>
-      <c r="P45" s="48"/>
-      <c r="Q45" s="48"/>
-      <c r="R45" s="49"/>
+      <c r="A45" s="35"/>
+      <c r="B45" s="34"/>
+      <c r="D45" s="80"/>
+      <c r="E45" s="81"/>
+      <c r="F45" s="102"/>
+      <c r="G45" s="103"/>
+      <c r="H45" s="103"/>
+      <c r="I45" s="103"/>
+      <c r="J45" s="103"/>
+      <c r="K45" s="103"/>
+      <c r="L45" s="30"/>
+      <c r="N45" s="80"/>
+      <c r="O45" s="66"/>
+      <c r="P45" s="66"/>
+      <c r="Q45" s="66"/>
+      <c r="R45" s="67"/>
     </row>
     <row r="46" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="107"/>
-      <c r="B46" s="28"/>
-      <c r="D46" s="44"/>
-      <c r="E46" s="45"/>
-      <c r="F46" s="46"/>
-      <c r="G46" s="47"/>
-      <c r="H46" s="47"/>
-      <c r="I46" s="47"/>
-      <c r="J46" s="47"/>
-      <c r="K46" s="47"/>
-      <c r="L46" s="39"/>
-      <c r="N46" s="44"/>
-      <c r="O46" s="48"/>
-      <c r="P46" s="48"/>
-      <c r="Q46" s="48"/>
-      <c r="R46" s="49"/>
+      <c r="A46" s="35"/>
+      <c r="B46" s="34"/>
+      <c r="D46" s="80"/>
+      <c r="E46" s="81"/>
+      <c r="F46" s="102"/>
+      <c r="G46" s="103"/>
+      <c r="H46" s="103"/>
+      <c r="I46" s="103"/>
+      <c r="J46" s="103"/>
+      <c r="K46" s="103"/>
+      <c r="L46" s="30"/>
+      <c r="N46" s="80"/>
+      <c r="O46" s="66"/>
+      <c r="P46" s="66"/>
+      <c r="Q46" s="66"/>
+      <c r="R46" s="67"/>
     </row>
     <row r="47" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="107"/>
-      <c r="B47" s="28"/>
-      <c r="D47" s="44"/>
-      <c r="E47" s="45"/>
-      <c r="F47" s="46"/>
-      <c r="G47" s="47"/>
-      <c r="H47" s="47"/>
-      <c r="I47" s="47"/>
-      <c r="J47" s="47"/>
-      <c r="K47" s="47"/>
-      <c r="L47" s="39"/>
-      <c r="N47" s="44"/>
-      <c r="O47" s="48"/>
-      <c r="P47" s="48"/>
-      <c r="Q47" s="48"/>
-      <c r="R47" s="49"/>
+      <c r="A47" s="35"/>
+      <c r="B47" s="34"/>
+      <c r="D47" s="80"/>
+      <c r="E47" s="81"/>
+      <c r="F47" s="102"/>
+      <c r="G47" s="103"/>
+      <c r="H47" s="103"/>
+      <c r="I47" s="103"/>
+      <c r="J47" s="103"/>
+      <c r="K47" s="103"/>
+      <c r="L47" s="30"/>
+      <c r="N47" s="80"/>
+      <c r="O47" s="66"/>
+      <c r="P47" s="66"/>
+      <c r="Q47" s="66"/>
+      <c r="R47" s="67"/>
     </row>
     <row r="48" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="107"/>
-      <c r="B48" s="28"/>
-      <c r="D48" s="44"/>
-      <c r="E48" s="45"/>
-      <c r="F48" s="46"/>
-      <c r="G48" s="47"/>
-      <c r="H48" s="47"/>
-      <c r="I48" s="47"/>
-      <c r="J48" s="47"/>
-      <c r="K48" s="47"/>
-      <c r="L48" s="39"/>
-      <c r="N48" s="44"/>
-      <c r="O48" s="48"/>
-      <c r="P48" s="48"/>
-      <c r="Q48" s="48"/>
-      <c r="R48" s="49"/>
+      <c r="A48" s="35"/>
+      <c r="B48" s="34"/>
+      <c r="D48" s="80"/>
+      <c r="E48" s="81"/>
+      <c r="F48" s="102"/>
+      <c r="G48" s="103"/>
+      <c r="H48" s="103"/>
+      <c r="I48" s="103"/>
+      <c r="J48" s="103"/>
+      <c r="K48" s="103"/>
+      <c r="L48" s="30"/>
+      <c r="N48" s="80"/>
+      <c r="O48" s="66"/>
+      <c r="P48" s="66"/>
+      <c r="Q48" s="66"/>
+      <c r="R48" s="67"/>
     </row>
     <row r="49" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="107"/>
-      <c r="B49" s="28"/>
-      <c r="D49" s="44"/>
-      <c r="E49" s="45"/>
-      <c r="F49" s="46"/>
-      <c r="G49" s="47"/>
-      <c r="H49" s="47"/>
-      <c r="I49" s="47"/>
-      <c r="J49" s="47"/>
-      <c r="K49" s="47"/>
-      <c r="L49" s="39"/>
-      <c r="N49" s="44"/>
-      <c r="O49" s="48"/>
-      <c r="P49" s="48"/>
-      <c r="Q49" s="48"/>
-      <c r="R49" s="49"/>
+      <c r="A49" s="35"/>
+      <c r="B49" s="34"/>
+      <c r="D49" s="80"/>
+      <c r="E49" s="81"/>
+      <c r="F49" s="102"/>
+      <c r="G49" s="103"/>
+      <c r="H49" s="103"/>
+      <c r="I49" s="103"/>
+      <c r="J49" s="103"/>
+      <c r="K49" s="103"/>
+      <c r="L49" s="30"/>
+      <c r="N49" s="80"/>
+      <c r="O49" s="66"/>
+      <c r="P49" s="66"/>
+      <c r="Q49" s="66"/>
+      <c r="R49" s="67"/>
     </row>
     <row r="50" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="107"/>
-      <c r="B50" s="28"/>
-      <c r="D50" s="44"/>
-      <c r="E50" s="45"/>
-      <c r="F50" s="46"/>
-      <c r="G50" s="47"/>
-      <c r="H50" s="47"/>
-      <c r="I50" s="47"/>
-      <c r="J50" s="47"/>
-      <c r="K50" s="47"/>
-      <c r="L50" s="40"/>
-      <c r="N50" s="44"/>
-      <c r="O50" s="48"/>
-      <c r="P50" s="48"/>
-      <c r="Q50" s="48"/>
-      <c r="R50" s="49"/>
+      <c r="A50" s="35"/>
+      <c r="B50" s="34"/>
+      <c r="D50" s="80"/>
+      <c r="E50" s="81"/>
+      <c r="F50" s="102"/>
+      <c r="G50" s="103"/>
+      <c r="H50" s="103"/>
+      <c r="I50" s="103"/>
+      <c r="J50" s="103"/>
+      <c r="K50" s="103"/>
+      <c r="L50" s="104"/>
+      <c r="N50" s="80"/>
+      <c r="O50" s="66"/>
+      <c r="P50" s="66"/>
+      <c r="Q50" s="66"/>
+      <c r="R50" s="67"/>
     </row>
     <row r="51" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="107"/>
-      <c r="B51" s="28"/>
-      <c r="D51" s="44"/>
-      <c r="E51" s="45"/>
-      <c r="F51" s="46"/>
-      <c r="G51" s="47"/>
-      <c r="H51" s="47"/>
-      <c r="I51" s="47"/>
-      <c r="J51" s="47"/>
-      <c r="K51" s="47"/>
-      <c r="L51" s="40"/>
-      <c r="N51" s="44"/>
-      <c r="O51" s="48"/>
-      <c r="P51" s="48"/>
-      <c r="Q51" s="48"/>
-      <c r="R51" s="49"/>
+      <c r="A51" s="35"/>
+      <c r="B51" s="34"/>
+      <c r="D51" s="80"/>
+      <c r="E51" s="81"/>
+      <c r="F51" s="102"/>
+      <c r="G51" s="103"/>
+      <c r="H51" s="103"/>
+      <c r="I51" s="103"/>
+      <c r="J51" s="103"/>
+      <c r="K51" s="103"/>
+      <c r="L51" s="104"/>
+      <c r="N51" s="80"/>
+      <c r="O51" s="66"/>
+      <c r="P51" s="66"/>
+      <c r="Q51" s="66"/>
+      <c r="R51" s="67"/>
     </row>
     <row r="52" spans="1:18" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="108"/>
-      <c r="B52" s="30"/>
-      <c r="D52" s="50"/>
-      <c r="E52" s="51"/>
-      <c r="F52" s="52"/>
-      <c r="G52" s="53"/>
-      <c r="H52" s="53"/>
-      <c r="I52" s="53"/>
-      <c r="J52" s="53"/>
-      <c r="K52" s="53"/>
-      <c r="L52" s="41"/>
-      <c r="N52" s="50"/>
-      <c r="O52" s="54"/>
-      <c r="P52" s="54"/>
-      <c r="Q52" s="54"/>
-      <c r="R52" s="55"/>
+      <c r="A52" s="36"/>
+      <c r="B52" s="95"/>
+      <c r="D52" s="88"/>
+      <c r="E52" s="89"/>
+      <c r="F52" s="105"/>
+      <c r="G52" s="106"/>
+      <c r="H52" s="106"/>
+      <c r="I52" s="106"/>
+      <c r="J52" s="106"/>
+      <c r="K52" s="106"/>
+      <c r="L52" s="107"/>
+      <c r="N52" s="88"/>
+      <c r="O52" s="91"/>
+      <c r="P52" s="91"/>
+      <c r="Q52" s="91"/>
+      <c r="R52" s="92"/>
     </row>
     <row r="53" spans="1:18" ht="14.1" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="155">
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="E3:F3"/>
-    <mergeCell ref="G3:I3"/>
-    <mergeCell ref="J3:L3"/>
-    <mergeCell ref="M3:Q3"/>
-    <mergeCell ref="R3:R7"/>
-    <mergeCell ref="G4:I4"/>
-    <mergeCell ref="J4:L4"/>
-    <mergeCell ref="M4:Q4"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="J9:L9"/>
-    <mergeCell ref="N9:O9"/>
-    <mergeCell ref="G10:I10"/>
-    <mergeCell ref="J10:L10"/>
-    <mergeCell ref="N10:O10"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:L5"/>
-    <mergeCell ref="A6:B7"/>
-    <mergeCell ref="D6:L7"/>
-    <mergeCell ref="G8:I8"/>
-    <mergeCell ref="J8:L8"/>
-    <mergeCell ref="P10:R10"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="J11:L11"/>
-    <mergeCell ref="N11:O11"/>
-    <mergeCell ref="P11:R11"/>
-    <mergeCell ref="G12:I12"/>
-    <mergeCell ref="J12:L12"/>
-    <mergeCell ref="N12:O12"/>
-    <mergeCell ref="P12:R12"/>
+    <mergeCell ref="D51:E51"/>
+    <mergeCell ref="F51:K51"/>
+    <mergeCell ref="N51:R51"/>
+    <mergeCell ref="D52:E52"/>
+    <mergeCell ref="F52:K52"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="F49:K49"/>
+    <mergeCell ref="N49:R49"/>
+    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="F50:K50"/>
+    <mergeCell ref="N50:R50"/>
+    <mergeCell ref="N52:R52"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="F47:K47"/>
+    <mergeCell ref="N47:R47"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="F48:K48"/>
+    <mergeCell ref="N48:R48"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="F45:K45"/>
+    <mergeCell ref="N45:R45"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="F46:K46"/>
+    <mergeCell ref="N46:R46"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="F43:K43"/>
+    <mergeCell ref="N43:R43"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="F44:K44"/>
+    <mergeCell ref="N44:R44"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="F41:K41"/>
+    <mergeCell ref="N41:R41"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="F42:K42"/>
+    <mergeCell ref="N42:R42"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="F39:K39"/>
+    <mergeCell ref="N39:R39"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="F40:K40"/>
+    <mergeCell ref="N40:R40"/>
+    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="F37:K37"/>
+    <mergeCell ref="N37:R37"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="F38:K38"/>
+    <mergeCell ref="N38:R38"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="F35:K35"/>
+    <mergeCell ref="N35:R35"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="F36:K36"/>
+    <mergeCell ref="N36:R36"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="F33:K33"/>
+    <mergeCell ref="N33:R33"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="F34:K34"/>
+    <mergeCell ref="N34:R34"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="F31:K31"/>
+    <mergeCell ref="N31:R31"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="F32:K32"/>
+    <mergeCell ref="N32:R32"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="F29:K29"/>
+    <mergeCell ref="N29:R29"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="F30:K30"/>
+    <mergeCell ref="N30:R30"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="F27:K27"/>
+    <mergeCell ref="N27:R27"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="F28:K28"/>
+    <mergeCell ref="N28:R28"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="F25:K25"/>
+    <mergeCell ref="N25:R25"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="F26:K26"/>
+    <mergeCell ref="N26:R26"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="F23:K23"/>
+    <mergeCell ref="N23:R23"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="F24:K24"/>
+    <mergeCell ref="N24:R24"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="F21:K21"/>
+    <mergeCell ref="N21:R21"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="F22:K22"/>
+    <mergeCell ref="N22:R22"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="D19:L19"/>
+    <mergeCell ref="N19:R19"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="F20:K20"/>
+    <mergeCell ref="N20:R20"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="J17:L17"/>
+    <mergeCell ref="N17:O17"/>
+    <mergeCell ref="P17:R17"/>
+    <mergeCell ref="G18:I18"/>
+    <mergeCell ref="J18:L18"/>
     <mergeCell ref="G15:I15"/>
     <mergeCell ref="J15:L15"/>
     <mergeCell ref="N15:O15"/>
@@ -2792,115 +2898,36 @@
     <mergeCell ref="J14:L14"/>
     <mergeCell ref="N14:O14"/>
     <mergeCell ref="P14:R14"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="D19:L19"/>
-    <mergeCell ref="N19:R19"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="F20:K20"/>
-    <mergeCell ref="N20:R20"/>
-    <mergeCell ref="G17:I17"/>
-    <mergeCell ref="J17:L17"/>
-    <mergeCell ref="N17:O17"/>
-    <mergeCell ref="P17:R17"/>
-    <mergeCell ref="G18:I18"/>
-    <mergeCell ref="J18:L18"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="F23:K23"/>
-    <mergeCell ref="N23:R23"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="F24:K24"/>
-    <mergeCell ref="N24:R24"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="F21:K21"/>
-    <mergeCell ref="N21:R21"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="F22:K22"/>
-    <mergeCell ref="N22:R22"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="F27:K27"/>
-    <mergeCell ref="N27:R27"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="F28:K28"/>
-    <mergeCell ref="N28:R28"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="F25:K25"/>
-    <mergeCell ref="N25:R25"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="F26:K26"/>
-    <mergeCell ref="N26:R26"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="F31:K31"/>
-    <mergeCell ref="N31:R31"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="F32:K32"/>
-    <mergeCell ref="N32:R32"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="F29:K29"/>
-    <mergeCell ref="N29:R29"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="F30:K30"/>
-    <mergeCell ref="N30:R30"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="F35:K35"/>
-    <mergeCell ref="N35:R35"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="F36:K36"/>
-    <mergeCell ref="N36:R36"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="F33:K33"/>
-    <mergeCell ref="N33:R33"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="F34:K34"/>
-    <mergeCell ref="N34:R34"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="F39:K39"/>
-    <mergeCell ref="N39:R39"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="F40:K40"/>
-    <mergeCell ref="N40:R40"/>
-    <mergeCell ref="D37:E37"/>
-    <mergeCell ref="F37:K37"/>
-    <mergeCell ref="N37:R37"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="F38:K38"/>
-    <mergeCell ref="N38:R38"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="F43:K43"/>
-    <mergeCell ref="N43:R43"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="F44:K44"/>
-    <mergeCell ref="N44:R44"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="F41:K41"/>
-    <mergeCell ref="N41:R41"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="F42:K42"/>
-    <mergeCell ref="N42:R42"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="F47:K47"/>
-    <mergeCell ref="N47:R47"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="F48:K48"/>
-    <mergeCell ref="N48:R48"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="F45:K45"/>
-    <mergeCell ref="N45:R45"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="F46:K46"/>
-    <mergeCell ref="N46:R46"/>
-    <mergeCell ref="D51:E51"/>
-    <mergeCell ref="F51:K51"/>
-    <mergeCell ref="N51:R51"/>
-    <mergeCell ref="D52:E52"/>
-    <mergeCell ref="F52:K52"/>
-    <mergeCell ref="D49:E49"/>
-    <mergeCell ref="F49:K49"/>
-    <mergeCell ref="N49:R49"/>
-    <mergeCell ref="D50:E50"/>
-    <mergeCell ref="F50:K50"/>
-    <mergeCell ref="N50:R50"/>
-    <mergeCell ref="N52:R52"/>
+    <mergeCell ref="P10:R10"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J11:L11"/>
+    <mergeCell ref="N11:O11"/>
+    <mergeCell ref="P11:R11"/>
+    <mergeCell ref="G12:I12"/>
+    <mergeCell ref="J12:L12"/>
+    <mergeCell ref="N12:O12"/>
+    <mergeCell ref="P12:R12"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="J9:L9"/>
+    <mergeCell ref="N9:O9"/>
+    <mergeCell ref="G10:I10"/>
+    <mergeCell ref="J10:L10"/>
+    <mergeCell ref="N10:O10"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:L5"/>
+    <mergeCell ref="A6:B7"/>
+    <mergeCell ref="D6:L7"/>
+    <mergeCell ref="G8:I8"/>
+    <mergeCell ref="J8:L8"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="G3:I3"/>
+    <mergeCell ref="J3:L3"/>
+    <mergeCell ref="M3:Q3"/>
+    <mergeCell ref="R3:R7"/>
+    <mergeCell ref="G4:I4"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="M4:Q4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>